<commit_message>
Sem 4 without EDR and Graph theory
</commit_message>
<xml_diff>
--- a/output/CGPA_Results.xlsx
+++ b/output/CGPA_Results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
   <si>
     <t>Rank</t>
   </si>
@@ -34,352 +34,355 @@
     <t>sem3</t>
   </si>
   <si>
+    <t>sem4</t>
+  </si>
+  <si>
     <t>CGPA</t>
   </si>
   <si>
     <t>JATHUNWATHTHA J.C.R.N.</t>
   </si>
   <si>
+    <t>ELAPATHA C.D.</t>
+  </si>
+  <si>
+    <t>NETTIKUMARA N.A.H.G.</t>
+  </si>
+  <si>
+    <t>ADIKARAM D.M.G.H.</t>
+  </si>
+  <si>
+    <t>PERERA G.M.B.</t>
+  </si>
+  <si>
+    <t>RATNAYAKE R.M.S.H.</t>
+  </si>
+  <si>
+    <t>DHANANJAYA K.T.G.T.N.</t>
+  </si>
+  <si>
     <t>PERERA W.A.L.S.</t>
   </si>
   <si>
-    <t>ELAPATHA C.D.</t>
-  </si>
-  <si>
-    <t>NETTIKUMARA N.A.H.G.</t>
-  </si>
-  <si>
-    <t>ADIKARAM D.M.G.H.</t>
+    <t>RATHNAYAKE M.A.G.K.N.</t>
+  </si>
+  <si>
+    <t>DISSANAYAKE G.R.G.K.</t>
+  </si>
+  <si>
+    <t>PERERA U.I.H.</t>
+  </si>
+  <si>
+    <t>KUMARASINGHE M.N.</t>
+  </si>
+  <si>
+    <t>WANIGASUNDARA W.M.H.</t>
   </si>
   <si>
     <t>BANDARA H.Y.W.</t>
   </si>
   <si>
+    <t>KUMARA K.B.R.</t>
+  </si>
+  <si>
+    <t>ILANKOON I.M.M.K.B.</t>
+  </si>
+  <si>
+    <t>KARIYAWASAM J.H.D.</t>
+  </si>
+  <si>
+    <t>IMADUWAGE O.N.H.</t>
+  </si>
+  <si>
+    <t>PERERA K.W.A.O.V.</t>
+  </si>
+  <si>
+    <t>SAMARASINGHE S.M.R.R.</t>
+  </si>
+  <si>
+    <t>GARUSINGHE S.B.</t>
+  </si>
+  <si>
+    <t>ARACHCHI A.D.I.D.</t>
+  </si>
+  <si>
+    <t>MALDENIYA P.A.D.G.R.</t>
+  </si>
+  <si>
+    <t>DISSANAYAKA D.M.D.P.</t>
+  </si>
+  <si>
+    <t>COLOMBAGE D.M.</t>
+  </si>
+  <si>
+    <t>DE MEL D.J.</t>
+  </si>
+  <si>
+    <t>FERNANDO W.H.D.</t>
+  </si>
+  <si>
+    <t>KARUNARATHNA G.K.T.</t>
+  </si>
+  <si>
+    <t>PEIRIS E.A.S.S.</t>
+  </si>
+  <si>
     <t>BANDARA W.D.A.C.</t>
   </si>
   <si>
-    <t>PERERA G.M.B.</t>
-  </si>
-  <si>
-    <t>RATNAYAKE R.M.S.H.</t>
-  </si>
-  <si>
-    <t>DHANANJAYA K.T.G.T.N.</t>
-  </si>
-  <si>
-    <t>COLOMBAGE D.M.</t>
-  </si>
-  <si>
-    <t>ILANKOON I.M.M.K.B.</t>
-  </si>
-  <si>
-    <t>KARIYAWASAM J.H.D.</t>
-  </si>
-  <si>
-    <t>KUMARA K.B.R.</t>
-  </si>
-  <si>
-    <t>RATHNAYAKE M.A.G.K.N.</t>
-  </si>
-  <si>
-    <t>DISSANAYAKE G.R.G.K.</t>
-  </si>
-  <si>
-    <t>PERERA K.W.A.O.V.</t>
-  </si>
-  <si>
-    <t>WANIGASUNDARA W.M.H.</t>
-  </si>
-  <si>
-    <t>KUMARASINGHE M.N.</t>
-  </si>
-  <si>
-    <t>PERERA U.I.H.</t>
-  </si>
-  <si>
-    <t>DE MEL D.J.</t>
-  </si>
-  <si>
-    <t>PEIRIS E.A.S.S.</t>
+    <t>RANASINGHE D.P.H.</t>
+  </si>
+  <si>
+    <t>KEERAWELLA K.P.C.P.</t>
   </si>
   <si>
     <t>RAHUL B.</t>
   </si>
   <si>
-    <t>DISSANAYAKA D.M.D.P.</t>
-  </si>
-  <si>
-    <t>IMADUWAGE O.N.H.</t>
-  </si>
-  <si>
-    <t>MALDENIYA P.A.D.G.R.</t>
-  </si>
-  <si>
-    <t>FERNANDO W.H.D.</t>
-  </si>
-  <si>
-    <t>SAMARASINGHE S.M.R.R.</t>
+    <t>CHANDRAKUMARA H.A.D.C.</t>
+  </si>
+  <si>
+    <t>WEDAMESTRIGE A.N.</t>
+  </si>
+  <si>
+    <t>AMARATHUNGE A.M.N.L.</t>
+  </si>
+  <si>
+    <t>GUNASEKARA L.U.A.</t>
+  </si>
+  <si>
+    <t>WIJESEKARA W.A.G.S.</t>
+  </si>
+  <si>
+    <t>RATHEESHAN A.R.</t>
+  </si>
+  <si>
+    <t>RASANJANA W.P.G.R.A.</t>
+  </si>
+  <si>
+    <t>GUNATHUNGA U.A.</t>
+  </si>
+  <si>
+    <t>DESHAN W.U.</t>
+  </si>
+  <si>
+    <t>ANTHONY C.S.B.</t>
+  </si>
+  <si>
+    <t>MUNASINGHE A.I.</t>
+  </si>
+  <si>
+    <t>PEIRIS T.S.R.</t>
+  </si>
+  <si>
+    <t>JAYAWEERA N.S.</t>
+  </si>
+  <si>
+    <t>DHARMAKEERTHI P.K.G.C.L.</t>
+  </si>
+  <si>
+    <t>WEERAKOON A.H.T.M.</t>
+  </si>
+  <si>
+    <t>KUMARA P.K.M.P.</t>
+  </si>
+  <si>
+    <t>PRIYADARSHANA S.A.D.</t>
+  </si>
+  <si>
+    <t>UPEKSHANI T.S.</t>
+  </si>
+  <si>
+    <t>DILHAN W.A.</t>
+  </si>
+  <si>
+    <t>PITIWADUGE D.N.</t>
   </si>
   <si>
     <t>PATHIRANA P.T.S.</t>
   </si>
   <si>
-    <t>RANASINGHE D.P.H.</t>
-  </si>
-  <si>
-    <t>GARUSINGHE S.B.</t>
-  </si>
-  <si>
-    <t>ARACHCHI A.D.I.D.</t>
-  </si>
-  <si>
-    <t>KEERAWELLA K.P.C.P.</t>
-  </si>
-  <si>
-    <t>KARUNARATHNA G.K.T.</t>
-  </si>
-  <si>
-    <t>DHARMAKEERTHI P.K.G.C.L.</t>
-  </si>
-  <si>
-    <t>WEERAKOON A.H.T.M.</t>
-  </si>
-  <si>
-    <t>RASANJANA W.P.G.R.A.</t>
-  </si>
-  <si>
-    <t>WEDAMESTRIGE A.N.</t>
-  </si>
-  <si>
-    <t>MUNASINGHE A.I.</t>
-  </si>
-  <si>
-    <t>CHANDRAKUMARA H.A.D.C.</t>
-  </si>
-  <si>
-    <t>WIJESEKARA W.A.G.S.</t>
-  </si>
-  <si>
-    <t>ANTHONY C.S.B.</t>
-  </si>
-  <si>
-    <t>AMARATHUNGE A.M.N.L.</t>
-  </si>
-  <si>
-    <t>DESHAN W.U.</t>
+    <t>KARUNANAYAKE A.H.D.</t>
+  </si>
+  <si>
+    <t>FERNANDO H.M.D.</t>
+  </si>
+  <si>
+    <t>PRISHMIKA H.W.N.</t>
+  </si>
+  <si>
+    <t>TENNAKOON U.G.R.B.</t>
+  </si>
+  <si>
+    <t>AROSHANA H.A.P.</t>
+  </si>
+  <si>
+    <t>GAMAGE SK</t>
+  </si>
+  <si>
+    <t>PERERA H.A.J.I.</t>
   </si>
   <si>
     <t>GUNASEKARA K.S.</t>
   </si>
   <si>
-    <t>GUNASEKARA L.U.A.</t>
-  </si>
-  <si>
-    <t>KARUNANAYAKE A.H.D.</t>
-  </si>
-  <si>
-    <t>JAYAWEERA N.S.</t>
-  </si>
-  <si>
-    <t>DILHAN W.A.</t>
-  </si>
-  <si>
-    <t>PERERA H.A.J.I.</t>
+    <t>RAHMAN M.F.A.</t>
+  </si>
+  <si>
+    <t>BALASOORIYA B.R.B.D.</t>
+  </si>
+  <si>
+    <t>UMAIR A.</t>
+  </si>
+  <si>
+    <t>RANATHUNGA R.J.K.O.H.</t>
+  </si>
+  <si>
+    <t>WEERASINGHE J.A.H.R.</t>
+  </si>
+  <si>
+    <t>WIJESINGHE U.G.S.K.D.</t>
+  </si>
+  <si>
+    <t>MEEDENIYA M.M.H.</t>
+  </si>
+  <si>
+    <t>PERAMUNAGE D.S.</t>
+  </si>
+  <si>
+    <t>ATHUKORALA U.R.</t>
+  </si>
+  <si>
+    <t>DILHARA D.S.</t>
+  </si>
+  <si>
+    <t>INDUWARA M.L.A.S.</t>
+  </si>
+  <si>
+    <t>WITHANAGE G.D.N.</t>
+  </si>
+  <si>
+    <t>DISSANAYAKE R.K.T.</t>
+  </si>
+  <si>
+    <t>SARUKA U.</t>
+  </si>
+  <si>
+    <t>ADHIKARI A.H.C.S.</t>
+  </si>
+  <si>
+    <t>RANAWAKA R.A.C.D.</t>
+  </si>
+  <si>
+    <t>ABISHEK L.</t>
+  </si>
+  <si>
+    <t>LENMINI B.L.W.</t>
+  </si>
+  <si>
+    <t>WIJESINGHE W.A.P.W.</t>
+  </si>
+  <si>
+    <t>RANAWAKA R.A.G.K.</t>
+  </si>
+  <si>
+    <t>ABEYWARDHANA T.C.W.</t>
+  </si>
+  <si>
+    <t>AYANAJA N.B.G.M.</t>
   </si>
   <si>
     <t>SHEHAN M.N.N.</t>
   </si>
   <si>
-    <t>AROSHANA H.A.P.</t>
-  </si>
-  <si>
-    <t>WEERASINGHE J.A.H.R.</t>
-  </si>
-  <si>
-    <t>RATHEESHAN A.R.</t>
-  </si>
-  <si>
-    <t>TENNAKOON U.G.R.B.</t>
-  </si>
-  <si>
-    <t>GUNATHUNGA U.A.</t>
-  </si>
-  <si>
-    <t>UPEKSHANI T.S.</t>
-  </si>
-  <si>
-    <t>PITIWADUGE D.N.</t>
-  </si>
-  <si>
-    <t>PRISHMIKA H.W.N.</t>
-  </si>
-  <si>
-    <t>FERNANDO H.M.D.</t>
-  </si>
-  <si>
-    <t>PRIYADARSHANA S.A.D.</t>
-  </si>
-  <si>
-    <t>PEIRIS T.S.R.</t>
-  </si>
-  <si>
-    <t>KUMARA P.K.M.P.</t>
-  </si>
-  <si>
-    <t>BALASOORIYA B.R.B.D.</t>
-  </si>
-  <si>
-    <t>RANATHUNGA R.J.K.O.H.</t>
-  </si>
-  <si>
-    <t>ATHUKORALA U.R.</t>
-  </si>
-  <si>
-    <t>DISSANAYAKE R.K.T.</t>
-  </si>
-  <si>
-    <t>RAHMAN M.F.A.</t>
-  </si>
-  <si>
-    <t>SARUKA U.</t>
-  </si>
-  <si>
-    <t>WIJESINGHE U.G.S.K.D.</t>
-  </si>
-  <si>
-    <t>ABISHEK L.</t>
-  </si>
-  <si>
-    <t>GAMAGE SK</t>
-  </si>
-  <si>
-    <t>RANAWAKA R.A.C.D.</t>
-  </si>
-  <si>
-    <t>UMAIR A.</t>
+    <t>KAUSHALYA R.G.S.P.</t>
+  </si>
+  <si>
+    <t>BANDARA K.M.N.D.</t>
+  </si>
+  <si>
+    <t>PRABHARSHA H.W.D.</t>
+  </si>
+  <si>
+    <t>NIRMANI W.T.</t>
   </si>
   <si>
     <t>ARACHCHIGE M. A. D. T. S.</t>
   </si>
   <si>
-    <t>WIJESINGHE W.A.P.W.</t>
-  </si>
-  <si>
-    <t>KAUSHALYA R.G.S.P.</t>
-  </si>
-  <si>
-    <t>ABEYWARDHANA T.C.W.</t>
-  </si>
-  <si>
-    <t>ADHIKARI A.H.C.S.</t>
-  </si>
-  <si>
-    <t>PERAMUNAGE D.S.</t>
-  </si>
-  <si>
-    <t>MEEDENIYA M.M.H.</t>
-  </si>
-  <si>
-    <t>DILHARA D.S.</t>
-  </si>
-  <si>
-    <t>BANDARA K.M.N.D.</t>
-  </si>
-  <si>
-    <t>PRABHARSHA H.W.D.</t>
-  </si>
-  <si>
-    <t>NIRMANI W.T.</t>
-  </si>
-  <si>
-    <t>INDUWARA M.L.A.S.</t>
-  </si>
-  <si>
-    <t>LENMINI B.L.W.</t>
-  </si>
-  <si>
-    <t>RANAWAKA R.A.G.K.</t>
+    <t>MANATUNGA K.D.</t>
+  </si>
+  <si>
+    <t>SAMARANAYAKA H.D.J.D.</t>
+  </si>
+  <si>
+    <t>UBEYSEKARA V.T.T.</t>
+  </si>
+  <si>
+    <t>PALIHENA H.H.</t>
+  </si>
+  <si>
+    <t>HANSINDU M.M.A.D.</t>
   </si>
   <si>
     <t>ABEYWARNA D.H.</t>
   </si>
   <si>
-    <t>PALIHENA H.H.</t>
-  </si>
-  <si>
-    <t>HANSINDU M.M.A.D.</t>
-  </si>
-  <si>
-    <t>WITHANAGE G.D.N.</t>
+    <t>ERANGA W.A.O.</t>
+  </si>
+  <si>
+    <t>GUNASEKARA H.M.</t>
+  </si>
+  <si>
+    <t>JAYASINGHE J.A.P.R.</t>
+  </si>
+  <si>
+    <t>RANASINGHE A.G.N.S.</t>
+  </si>
+  <si>
+    <t>AMARASINGHE A.A.D.K.</t>
+  </si>
+  <si>
+    <t>SAMARASEKARA S.M.R.P.</t>
+  </si>
+  <si>
+    <t>THARUSHIKA G.K.E.</t>
+  </si>
+  <si>
+    <t>PIYUMAL N.P.P.</t>
+  </si>
+  <si>
+    <t>SANTHOSH S.</t>
+  </si>
+  <si>
+    <t>AHAMED A.M.S.</t>
   </si>
   <si>
     <t>HIMASARA W.V.M.J.</t>
   </si>
   <si>
-    <t>AYANAJA N.B.G.M.</t>
-  </si>
-  <si>
-    <t>UBEYSEKARA V.T.T.</t>
-  </si>
-  <si>
-    <t>GUNASEKARA H.M.</t>
-  </si>
-  <si>
-    <t>ERANGA W.A.O.</t>
-  </si>
-  <si>
-    <t>RANASINGHE A.G.N.S.</t>
-  </si>
-  <si>
-    <t>SAMARANAYAKA H.D.J.D.</t>
-  </si>
-  <si>
-    <t>JAYASINGHE J.A.P.R.</t>
+    <t>HAKAM M.R.A.</t>
   </si>
   <si>
     <t>IMBULPITIYA B.N.</t>
   </si>
   <si>
-    <t>MANATUNGA K.D.</t>
-  </si>
-  <si>
-    <t>AHAMED A.M.S.</t>
-  </si>
-  <si>
-    <t>AMARASINGHE A.A.D.K.</t>
-  </si>
-  <si>
-    <t>THARUSHIKA G.K.E.</t>
-  </si>
-  <si>
-    <t>HAKAM M.R.A.</t>
-  </si>
-  <si>
-    <t>SANTHOSH S.</t>
-  </si>
-  <si>
     <t>JAYAKODY J.A.C.P.</t>
   </si>
   <si>
-    <t>SAMARASEKARA S.M.R.P.</t>
+    <t>NUWANAKA W.A.S.</t>
   </si>
   <si>
     <t>HENDENIYA H.M.J.C.</t>
   </si>
   <si>
-    <t>PIYUMAL N.P.P.</t>
+    <t>WIJETHILAKA J.S.</t>
+  </si>
+  <si>
+    <t>FERNANDO LTJ</t>
   </si>
   <si>
     <t>GUNARATHNA K.T.M.B.</t>
-  </si>
-  <si>
-    <t>NUWANAKA W.A.S.</t>
-  </si>
-  <si>
-    <t>WIJETHILAKA J.S.</t>
-  </si>
-  <si>
-    <t>FERNANDO LTJ</t>
   </si>
 </sst>
 </file>
@@ -711,10 +714,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -736,8 +739,11 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
@@ -745,7 +751,7 @@
         <v>230266</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -759,16 +765,19 @@
       <c r="G2">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>230487</v>
+        <v>230171</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3">
         <v>4</v>
@@ -777,67 +786,76 @@
         <v>4</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>3.973</v>
       </c>
       <c r="G3">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3">
+        <v>3.993</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>230171</v>
+        <v>230436</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4">
         <v>4</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>3.973</v>
       </c>
       <c r="F4">
-        <v>3.973</v>
+        <v>4</v>
       </c>
       <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>3.993</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>230018</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>3.96</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
         <v>3.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>230436</v>
-      </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="E5">
-        <v>3.973</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>3.99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>230018</v>
+        <v>230476</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -849,18 +867,21 @@
         <v>3.96</v>
       </c>
       <c r="G6">
-        <v>3.985</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>230074</v>
+        <v>230548</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -872,18 +893,21 @@
         <v>3.96</v>
       </c>
       <c r="G7">
-        <v>3.985</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H7">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>230082</v>
+        <v>230138</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -892,21 +916,24 @@
         <v>4</v>
       </c>
       <c r="F8">
-        <v>3.96</v>
+        <v>3.957</v>
       </c>
       <c r="G8">
-        <v>3.985</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>3.989</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>230476</v>
+        <v>230487</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -915,21 +942,24 @@
         <v>4</v>
       </c>
       <c r="F9">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>3.985</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H9">
+        <v>3.984</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>230548</v>
+        <v>230544</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -938,67 +968,76 @@
         <v>4</v>
       </c>
       <c r="F10">
-        <v>3.96</v>
+        <v>3.921</v>
       </c>
       <c r="G10">
-        <v>3.985</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H10">
+        <v>3.98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>230138</v>
+        <v>230159</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D11">
         <v>4</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>3.955</v>
       </c>
       <c r="F11">
-        <v>3.957</v>
+        <v>3.954</v>
       </c>
       <c r="G11">
-        <v>3.984</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H11">
+        <v>3.977</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
-        <v>230108</v>
+        <v>230486</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D12">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E12">
         <v>4</v>
       </c>
       <c r="F12">
-        <v>3.954</v>
+        <v>3.907</v>
       </c>
       <c r="G12">
-        <v>3.97</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H12">
+        <v>3.976</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
-        <v>230256</v>
+        <v>230355</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D13">
         <v>4</v>
@@ -1007,21 +1046,24 @@
         <v>4</v>
       </c>
       <c r="F13">
-        <v>3.925</v>
+        <v>3.9</v>
       </c>
       <c r="G13">
-        <v>3.97</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H13">
+        <v>3.975</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
-        <v>230318</v>
+        <v>230680</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D14">
         <v>4</v>
@@ -1030,24 +1072,27 @@
         <v>4</v>
       </c>
       <c r="F14">
-        <v>3.924</v>
+        <v>3.9</v>
       </c>
       <c r="G14">
-        <v>3.97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H14">
+        <v>3.975</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
-        <v>230352</v>
+        <v>230074</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D15">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E15">
         <v>4</v>
@@ -1056,202 +1101,229 @@
         <v>3.96</v>
       </c>
       <c r="G15">
-        <v>3.969</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H15">
+        <v>3.974</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16">
-        <v>230544</v>
+        <v>230352</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E16">
         <v>4</v>
       </c>
       <c r="F16">
-        <v>3.921</v>
+        <v>3.96</v>
       </c>
       <c r="G16">
-        <v>3.969</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H16">
+        <v>3.973</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17">
-        <v>230159</v>
+        <v>230256</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17">
         <v>4</v>
       </c>
       <c r="E17">
-        <v>3.955</v>
+        <v>4</v>
       </c>
       <c r="F17">
-        <v>3.954</v>
+        <v>3.925</v>
       </c>
       <c r="G17">
+        <v>3.936</v>
+      </c>
+      <c r="H17">
         <v>3.965</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:8">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18">
-        <v>230481</v>
+        <v>230318</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D18">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E18">
         <v>4</v>
       </c>
       <c r="F18">
-        <v>4</v>
+        <v>3.924</v>
       </c>
       <c r="G18">
+        <v>3.936</v>
+      </c>
+      <c r="H18">
         <v>3.965</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:8">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19">
-        <v>230680</v>
+        <v>230258</v>
       </c>
       <c r="C19" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E19">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F19">
-        <v>3.9</v>
+        <v>3.957</v>
       </c>
       <c r="G19">
+        <v>4</v>
+      </c>
+      <c r="H19">
         <v>3.963</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:8">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20">
-        <v>230355</v>
+        <v>230481</v>
       </c>
       <c r="C20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D20">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E20">
         <v>4</v>
       </c>
       <c r="F20">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>3.961</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H20">
+        <v>3.962</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21">
-        <v>230486</v>
+        <v>230566</v>
       </c>
       <c r="C21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D21">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E21">
         <v>4</v>
       </c>
       <c r="F21">
-        <v>3.907</v>
+        <v>3.884</v>
       </c>
       <c r="G21">
-        <v>3.961</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H21">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22">
-        <v>230121</v>
+        <v>230197</v>
       </c>
       <c r="C22" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D22">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E22">
-        <v>4</v>
+        <v>3.934</v>
       </c>
       <c r="F22">
-        <v>3.921</v>
+        <v>3.899</v>
       </c>
       <c r="G22">
-        <v>3.96</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H22">
+        <v>3.958</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23">
-        <v>230469</v>
+        <v>230051</v>
       </c>
       <c r="C23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D23">
         <v>4</v>
       </c>
       <c r="E23">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F23">
-        <v>3.937</v>
+        <v>3.83</v>
       </c>
       <c r="G23">
-        <v>3.96</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H23">
+        <v>3.957</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24">
-        <v>230508</v>
+        <v>230390</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D24">
         <v>4</v>
@@ -1260,13 +1332,16 @@
         <v>4</v>
       </c>
       <c r="F24">
-        <v>3.882</v>
+        <v>3.873</v>
       </c>
       <c r="G24">
-        <v>3.955</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+        <v>3.952</v>
+      </c>
+      <c r="H24">
+        <v>3.956</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1274,7 +1349,7 @@
         <v>230155</v>
       </c>
       <c r="C25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D25">
         <v>4</v>
@@ -1286,56 +1361,65 @@
         <v>3.957</v>
       </c>
       <c r="G25">
-        <v>3.953</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+        <v>3.942</v>
+      </c>
+      <c r="H25">
+        <v>3.955</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26">
-        <v>230258</v>
+        <v>230108</v>
       </c>
       <c r="C26" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D26">
         <v>3.935</v>
       </c>
       <c r="E26">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F26">
-        <v>3.957</v>
+        <v>3.954</v>
       </c>
       <c r="G26">
+        <v>3.925</v>
+      </c>
+      <c r="H26">
         <v>3.953</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:8">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27">
-        <v>230390</v>
+        <v>230121</v>
       </c>
       <c r="C27" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D27">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E27">
         <v>4</v>
       </c>
       <c r="F27">
-        <v>3.873</v>
+        <v>3.921</v>
       </c>
       <c r="G27">
-        <v>3.951</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H27">
+        <v>3.953</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1343,7 +1427,7 @@
         <v>230186</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D28">
         <v>4</v>
@@ -1355,64 +1439,73 @@
         <v>3.869</v>
       </c>
       <c r="G28">
-        <v>3.95</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+        <v>3.942</v>
+      </c>
+      <c r="H28">
+        <v>3.952</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29">
-        <v>230566</v>
+        <v>230322</v>
       </c>
       <c r="C29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D29">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E29">
-        <v>4</v>
+        <v>3.908</v>
       </c>
       <c r="F29">
-        <v>3.884</v>
+        <v>3.9</v>
       </c>
       <c r="G29">
-        <v>3.942</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H29">
+        <v>3.952</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30">
-        <v>230468</v>
+        <v>230469</v>
       </c>
       <c r="C30" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D30">
+        <v>4</v>
+      </c>
+      <c r="E30">
+        <v>3.96</v>
+      </c>
+      <c r="F30">
+        <v>3.937</v>
+      </c>
+      <c r="G30">
         <v>3.914</v>
       </c>
-      <c r="E30">
-        <v>4</v>
-      </c>
-      <c r="F30">
-        <v>3.895</v>
-      </c>
-      <c r="G30">
-        <v>3.94</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="H30">
+        <v>3.952</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31">
-        <v>230521</v>
+        <v>230082</v>
       </c>
       <c r="C31" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D31">
         <v>4</v>
@@ -1421,44 +1514,50 @@
         <v>4</v>
       </c>
       <c r="F31">
-        <v>3.843</v>
+        <v>3.96</v>
       </c>
       <c r="G31">
-        <v>3.94</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+        <v>3.842</v>
+      </c>
+      <c r="H31">
+        <v>3.95</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32">
-        <v>230197</v>
+        <v>230521</v>
       </c>
       <c r="C32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32">
         <v>4</v>
       </c>
       <c r="E32">
-        <v>3.934</v>
+        <v>4</v>
       </c>
       <c r="F32">
-        <v>3.899</v>
+        <v>3.843</v>
       </c>
       <c r="G32">
-        <v>3.936</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+        <v>3.959</v>
+      </c>
+      <c r="H32">
+        <v>3.95</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33">
-        <v>230051</v>
+        <v>230332</v>
       </c>
       <c r="C33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D33">
         <v>4</v>
@@ -1467,21 +1566,24 @@
         <v>4</v>
       </c>
       <c r="F33">
-        <v>3.83</v>
+        <v>3.79</v>
       </c>
       <c r="G33">
-        <v>3.935</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H33">
+        <v>3.947</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34">
-        <v>230332</v>
+        <v>230508</v>
       </c>
       <c r="C34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -1490,67 +1592,76 @@
         <v>4</v>
       </c>
       <c r="F34">
-        <v>3.79</v>
+        <v>3.882</v>
       </c>
       <c r="G34">
-        <v>3.931</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
+        <v>3.852</v>
+      </c>
+      <c r="H34">
+        <v>3.933</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35">
-        <v>230322</v>
+        <v>230100</v>
       </c>
       <c r="C35" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D35">
         <v>4</v>
       </c>
       <c r="E35">
-        <v>3.908</v>
+        <v>4</v>
       </c>
       <c r="F35">
-        <v>3.9</v>
+        <v>3.721</v>
       </c>
       <c r="G35">
-        <v>3.926</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H35">
+        <v>3.914</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36">
-        <v>230140</v>
+        <v>230687</v>
       </c>
       <c r="C36" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D36">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E36">
-        <v>3.96</v>
+        <v>3.934</v>
       </c>
       <c r="F36">
-        <v>3.873</v>
+        <v>3.83</v>
       </c>
       <c r="G36">
-        <v>3.921</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
+        <v>3.876</v>
+      </c>
+      <c r="H36">
+        <v>3.909</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37">
-        <v>230689</v>
+        <v>230038</v>
       </c>
       <c r="C37" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -1559,159 +1670,180 @@
         <v>4</v>
       </c>
       <c r="F37">
-        <v>3.771</v>
+        <v>3.691</v>
       </c>
       <c r="G37">
-        <v>3.917</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
+        <v>3.914</v>
+      </c>
+      <c r="H37">
+        <v>3.901</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38">
-        <v>230536</v>
+        <v>230212</v>
       </c>
       <c r="C38" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D38">
         <v>3.957</v>
       </c>
       <c r="E38">
-        <v>3.96</v>
+        <v>3.882</v>
       </c>
       <c r="F38">
-        <v>3.847</v>
+        <v>3.821</v>
       </c>
       <c r="G38">
-        <v>3.916</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H38">
+        <v>3.899</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39">
-        <v>230687</v>
+        <v>230724</v>
       </c>
       <c r="C39" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D39">
         <v>4</v>
       </c>
       <c r="E39">
-        <v>3.934</v>
+        <v>3.869</v>
       </c>
       <c r="F39">
-        <v>3.83</v>
+        <v>3.847</v>
       </c>
       <c r="G39">
-        <v>3.909</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+        <v>3.873</v>
+      </c>
+      <c r="H39">
+        <v>3.897</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40">
-        <v>230417</v>
+        <v>230539</v>
       </c>
       <c r="C40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D40">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E40">
-        <v>3.939</v>
+        <v>4</v>
       </c>
       <c r="F40">
-        <v>3.804</v>
+        <v>3.652</v>
       </c>
       <c r="G40">
-        <v>3.901</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H40">
+        <v>3.896</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41">
-        <v>230100</v>
+        <v>230536</v>
       </c>
       <c r="C41" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D41">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E41">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F41">
-        <v>3.721</v>
+        <v>3.847</v>
       </c>
       <c r="G41">
+        <v>3.809</v>
+      </c>
+      <c r="H41">
         <v>3.893</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:8">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42">
-        <v>230724</v>
+        <v>230218</v>
       </c>
       <c r="C42" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D42">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E42">
-        <v>3.869</v>
+        <v>3.811</v>
       </c>
       <c r="F42">
-        <v>3.847</v>
+        <v>3.825</v>
       </c>
       <c r="G42">
-        <v>3.891</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H42">
+        <v>3.892</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43">
-        <v>230045</v>
+        <v>230130</v>
       </c>
       <c r="C43" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D43">
         <v>4</v>
       </c>
       <c r="E43">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F43">
-        <v>3.704</v>
+        <v>3.714</v>
       </c>
       <c r="G43">
-        <v>3.886</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
+        <v>3.889</v>
+      </c>
+      <c r="H43">
+        <v>3.89</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44">
-        <v>230038</v>
+        <v>230045</v>
       </c>
       <c r="C44" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D44">
         <v>4</v>
@@ -1720,473 +1852,536 @@
         <v>4</v>
       </c>
       <c r="F44">
-        <v>3.691</v>
+        <v>3.704</v>
       </c>
       <c r="G44">
-        <v>3.881</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
+        <v>3.852</v>
+      </c>
+      <c r="H44">
+        <v>3.889</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45">
-        <v>230130</v>
+        <v>230417</v>
       </c>
       <c r="C45" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D45">
         <v>4</v>
       </c>
       <c r="E45">
-        <v>3.96</v>
+        <v>3.939</v>
       </c>
       <c r="F45">
-        <v>3.714</v>
+        <v>3.804</v>
       </c>
       <c r="G45">
-        <v>3.881</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
+        <v>3.789</v>
+      </c>
+      <c r="H45">
+        <v>3.883</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46">
-        <v>230211</v>
+        <v>230470</v>
       </c>
       <c r="C46" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D46">
         <v>4</v>
       </c>
       <c r="E46">
-        <v>3.895</v>
+        <v>4</v>
       </c>
       <c r="F46">
-        <v>3.782</v>
+        <v>3.526</v>
       </c>
       <c r="G46">
-        <v>3.876</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H46">
+        <v>3.881</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47">
-        <v>230212</v>
+        <v>230300</v>
       </c>
       <c r="C47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D47">
-        <v>3.957</v>
+        <v>3.935</v>
       </c>
       <c r="E47">
-        <v>3.882</v>
+        <v>4</v>
       </c>
       <c r="F47">
-        <v>3.821</v>
+        <v>3.713</v>
       </c>
       <c r="G47">
-        <v>3.876</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
+        <v>3.873</v>
+      </c>
+      <c r="H47">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48">
-        <v>230321</v>
+        <v>230140</v>
       </c>
       <c r="C48" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D48">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E48">
-        <v>3.947</v>
+        <v>3.96</v>
       </c>
       <c r="F48">
-        <v>3.73</v>
+        <v>3.873</v>
       </c>
       <c r="G48">
-        <v>3.876</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
+        <v>3.742</v>
+      </c>
+      <c r="H48">
+        <v>3.877</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49">
-        <v>230300</v>
+        <v>230689</v>
       </c>
       <c r="C49" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D49">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E49">
         <v>4</v>
       </c>
       <c r="F49">
-        <v>3.713</v>
+        <v>3.771</v>
       </c>
       <c r="G49">
-        <v>3.875</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
+        <v>3.709</v>
+      </c>
+      <c r="H49">
+        <v>3.87</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50">
-        <v>230145</v>
+        <v>230353</v>
       </c>
       <c r="C50" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D50">
-        <v>3.935</v>
+        <v>3.9</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F50">
-        <v>3.704</v>
+        <v>3.613</v>
       </c>
       <c r="G50">
-        <v>3.871</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H50">
+        <v>3.868</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51">
-        <v>230477</v>
+        <v>230502</v>
       </c>
       <c r="C51" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D51">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E51">
-        <v>3.817</v>
+        <v>3.947</v>
       </c>
       <c r="F51">
-        <v>3.873</v>
+        <v>3.586</v>
       </c>
       <c r="G51">
-        <v>3.866</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H51">
+        <v>3.867</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52">
-        <v>230613</v>
+        <v>230659</v>
       </c>
       <c r="C52" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D52">
-        <v>4</v>
+        <v>3.857</v>
       </c>
       <c r="E52">
-        <v>3.947</v>
+        <v>3.869</v>
       </c>
       <c r="F52">
-        <v>3.699</v>
+        <v>3.804</v>
       </c>
       <c r="G52">
-        <v>3.865</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H52">
+        <v>3.866</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53">
-        <v>230058</v>
+        <v>230145</v>
       </c>
       <c r="C53" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D53">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E53">
-        <v>3.908</v>
+        <v>4</v>
       </c>
       <c r="F53">
-        <v>3.713</v>
+        <v>3.704</v>
       </c>
       <c r="G53">
-        <v>3.855</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7">
+        <v>3.809</v>
+      </c>
+      <c r="H53">
+        <v>3.862</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54">
-        <v>230697</v>
+        <v>230492</v>
       </c>
       <c r="C54" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D54">
-        <v>3.957</v>
+        <v>3.935</v>
       </c>
       <c r="E54">
-        <v>3.96</v>
+        <v>3.908</v>
       </c>
       <c r="F54">
-        <v>3.671</v>
+        <v>3.69</v>
       </c>
       <c r="G54">
-        <v>3.855</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7">
+        <v>3.914</v>
+      </c>
+      <c r="H54">
+        <v>3.861</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55">
-        <v>230539</v>
+        <v>230468</v>
       </c>
       <c r="C55" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D55">
-        <v>3.935</v>
+        <v>3.914</v>
       </c>
       <c r="E55">
         <v>4</v>
       </c>
       <c r="F55">
-        <v>3.652</v>
+        <v>3.895</v>
       </c>
       <c r="G55">
-        <v>3.851</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
+        <v>3.594</v>
+      </c>
+      <c r="H55">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56">
-        <v>230629</v>
+        <v>230321</v>
       </c>
       <c r="C56" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D56">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E56">
-        <v>3.908</v>
+        <v>3.947</v>
       </c>
       <c r="F56">
-        <v>3.726</v>
+        <v>3.73</v>
       </c>
       <c r="G56">
-        <v>3.85</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7">
+        <v>3.704</v>
+      </c>
+      <c r="H56">
+        <v>3.845</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57">
-        <v>230218</v>
+        <v>230180</v>
       </c>
       <c r="C57" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D57">
         <v>3.935</v>
       </c>
       <c r="E57">
-        <v>3.811</v>
+        <v>3.817</v>
       </c>
       <c r="F57">
-        <v>3.825</v>
+        <v>3.778</v>
       </c>
       <c r="G57">
-        <v>3.844</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7">
+        <v>3.842</v>
+      </c>
+      <c r="H57">
+        <v>3.843</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58">
-        <v>230659</v>
+        <v>230500</v>
       </c>
       <c r="C58" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D58">
-        <v>3.857</v>
+        <v>3.957</v>
       </c>
       <c r="E58">
-        <v>3.869</v>
+        <v>3.908</v>
       </c>
       <c r="F58">
-        <v>3.804</v>
+        <v>3.678</v>
       </c>
       <c r="G58">
-        <v>3.841</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7">
+        <v>3.826</v>
+      </c>
+      <c r="H58">
+        <v>3.842</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59">
-        <v>230492</v>
+        <v>230629</v>
       </c>
       <c r="C59" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D59">
-        <v>3.935</v>
+        <v>3.957</v>
       </c>
       <c r="E59">
         <v>3.908</v>
       </c>
       <c r="F59">
-        <v>3.69</v>
+        <v>3.726</v>
       </c>
       <c r="G59">
-        <v>3.836</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
+        <v>3.771</v>
+      </c>
+      <c r="H59">
+        <v>3.84</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60">
-        <v>230500</v>
+        <v>230058</v>
       </c>
       <c r="C60" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D60">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E60">
         <v>3.908</v>
       </c>
       <c r="F60">
-        <v>3.678</v>
+        <v>3.713</v>
       </c>
       <c r="G60">
-        <v>3.831</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
+        <v>3.726</v>
+      </c>
+      <c r="H60">
+        <v>3.836</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61">
-        <v>230180</v>
+        <v>230195</v>
       </c>
       <c r="C61" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D61">
-        <v>3.935</v>
+        <v>3.957</v>
       </c>
       <c r="E61">
-        <v>3.817</v>
+        <v>3.791</v>
       </c>
       <c r="F61">
-        <v>3.778</v>
+        <v>3.678</v>
       </c>
       <c r="G61">
-        <v>3.83</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7">
+        <v>3.914</v>
+      </c>
+      <c r="H61">
+        <v>3.834</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62">
-        <v>230502</v>
+        <v>230477</v>
       </c>
       <c r="C62" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D62">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E62">
-        <v>3.947</v>
+        <v>3.817</v>
       </c>
       <c r="F62">
-        <v>3.586</v>
+        <v>3.873</v>
       </c>
       <c r="G62">
-        <v>3.821</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7">
+        <v>3.704</v>
+      </c>
+      <c r="H62">
+        <v>3.832</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63">
-        <v>230470</v>
+        <v>230211</v>
       </c>
       <c r="C63" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D63">
         <v>4</v>
       </c>
       <c r="E63">
-        <v>4</v>
+        <v>3.895</v>
       </c>
       <c r="F63">
-        <v>3.526</v>
+        <v>3.782</v>
       </c>
       <c r="G63">
-        <v>3.818</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7">
+        <v>3.647</v>
+      </c>
+      <c r="H63">
+        <v>3.831</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64">
-        <v>230353</v>
+        <v>230507</v>
       </c>
       <c r="C64" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D64">
+        <v>3.857</v>
+      </c>
+      <c r="E64">
+        <v>3.877</v>
+      </c>
+      <c r="F64">
+        <v>3.645</v>
+      </c>
+      <c r="G64">
         <v>3.9</v>
       </c>
-      <c r="E64">
-        <v>3.96</v>
-      </c>
-      <c r="F64">
-        <v>3.613</v>
-      </c>
-      <c r="G64">
-        <v>3.813</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7">
+      <c r="H64">
+        <v>3.819</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2194,7 +2389,7 @@
         <v>230070</v>
       </c>
       <c r="C65" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D65">
         <v>3.957</v>
@@ -2206,746 +2401,845 @@
         <v>3.717</v>
       </c>
       <c r="G65">
-        <v>3.808</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7">
+        <v>3.789</v>
+      </c>
+      <c r="H65">
+        <v>3.817</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66">
-        <v>230525</v>
+        <v>230654</v>
       </c>
       <c r="C66" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D66">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E66">
-        <v>4</v>
+        <v>3.839</v>
       </c>
       <c r="F66">
-        <v>3.5</v>
+        <v>3.591</v>
       </c>
       <c r="G66">
-        <v>3.808</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7">
+        <v>3.871</v>
+      </c>
+      <c r="H66">
+        <v>3.809</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67">
-        <v>230063</v>
+        <v>230525</v>
       </c>
       <c r="C67" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D67">
         <v>4</v>
       </c>
       <c r="E67">
-        <v>3.908</v>
+        <v>4</v>
       </c>
       <c r="F67">
-        <v>3.56</v>
+        <v>3.5</v>
       </c>
       <c r="G67">
-        <v>3.796</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7">
+        <v>3.726</v>
+      </c>
+      <c r="H67">
+        <v>3.806</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68">
-        <v>230164</v>
+        <v>230697</v>
       </c>
       <c r="C68" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D68">
         <v>3.957</v>
       </c>
       <c r="E68">
-        <v>3.869</v>
+        <v>3.96</v>
       </c>
       <c r="F68">
-        <v>3.626</v>
+        <v>3.671</v>
       </c>
       <c r="G68">
-        <v>3.796</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
+        <v>3.633</v>
+      </c>
+      <c r="H68">
+        <v>3.805</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69">
-        <v>230507</v>
+        <v>230726</v>
       </c>
       <c r="C69" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D69">
-        <v>3.857</v>
+        <v>3.892</v>
       </c>
       <c r="E69">
-        <v>3.877</v>
+        <v>3.869</v>
       </c>
       <c r="F69">
-        <v>3.645</v>
+        <v>3.66</v>
       </c>
       <c r="G69">
-        <v>3.796</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7">
+        <v>3.789</v>
+      </c>
+      <c r="H69">
+        <v>3.802</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70">
-        <v>230585</v>
+        <v>230407</v>
       </c>
       <c r="C70" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D70">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E70">
-        <v>3.96</v>
+        <v>3.756</v>
       </c>
       <c r="F70">
-        <v>3.543</v>
+        <v>3.508</v>
       </c>
       <c r="G70">
-        <v>3.795</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H70">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71">
-        <v>230726</v>
+        <v>230473</v>
       </c>
       <c r="C71" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D71">
         <v>3.892</v>
       </c>
       <c r="E71">
-        <v>3.869</v>
+        <v>3.908</v>
       </c>
       <c r="F71">
-        <v>3.66</v>
+        <v>3.443</v>
       </c>
       <c r="G71">
-        <v>3.795</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H71">
+        <v>3.794</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72">
-        <v>230016</v>
+        <v>230063</v>
       </c>
       <c r="C72" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D72">
         <v>4</v>
       </c>
       <c r="E72">
-        <v>3.911</v>
+        <v>3.908</v>
       </c>
       <c r="F72">
-        <v>3.479</v>
+        <v>3.56</v>
       </c>
       <c r="G72">
-        <v>3.79</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7">
+        <v>3.705</v>
+      </c>
+      <c r="H72">
+        <v>3.793</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73">
-        <v>230195</v>
+        <v>230147</v>
       </c>
       <c r="C73" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D73">
-        <v>3.957</v>
+        <v>3.892</v>
       </c>
       <c r="E73">
-        <v>3.791</v>
+        <v>3.817</v>
       </c>
       <c r="F73">
-        <v>3.678</v>
+        <v>3.508</v>
       </c>
       <c r="G73">
-        <v>3.786</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H73">
+        <v>3.788</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74">
-        <v>230526</v>
+        <v>230261</v>
       </c>
       <c r="C74" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D74">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E74">
-        <v>3.947</v>
+        <v>3.747</v>
       </c>
       <c r="F74">
-        <v>3.495</v>
+        <v>3.458</v>
       </c>
       <c r="G74">
-        <v>3.771</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H74">
+        <v>3.785</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75">
-        <v>230654</v>
+        <v>230735</v>
       </c>
       <c r="C75" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D75">
         <v>3.935</v>
       </c>
       <c r="E75">
-        <v>3.839</v>
+        <v>3.786</v>
       </c>
       <c r="F75">
-        <v>3.591</v>
+        <v>3.399</v>
       </c>
       <c r="G75">
-        <v>3.766</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7">
+        <v>4</v>
+      </c>
+      <c r="H75">
+        <v>3.78</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76">
-        <v>230052</v>
+        <v>230164</v>
       </c>
       <c r="C76" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D76">
-        <v>3.75</v>
+        <v>3.957</v>
       </c>
       <c r="E76">
-        <v>3.844</v>
+        <v>3.869</v>
       </c>
       <c r="F76">
-        <v>3.63</v>
+        <v>3.626</v>
       </c>
       <c r="G76">
-        <v>3.752</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7">
+        <v>3.666</v>
+      </c>
+      <c r="H76">
+        <v>3.779</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77">
-        <v>230727</v>
+        <v>230585</v>
       </c>
       <c r="C77" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D77">
-        <v>3.785</v>
+        <v>3.935</v>
       </c>
       <c r="E77">
-        <v>3.888</v>
+        <v>3.96</v>
       </c>
       <c r="F77">
-        <v>3.54</v>
+        <v>3.543</v>
       </c>
       <c r="G77">
-        <v>3.75</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7">
+        <v>3.676</v>
+      </c>
+      <c r="H77">
+        <v>3.778</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78">
-        <v>230327</v>
+        <v>230017</v>
       </c>
       <c r="C78" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D78">
-        <v>3.85</v>
+        <v>3.9</v>
       </c>
       <c r="E78">
-        <v>3.656</v>
+        <v>3.947</v>
       </c>
       <c r="F78">
-        <v>3.765</v>
+        <v>3.441</v>
       </c>
       <c r="G78">
-        <v>3.743</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7">
+        <v>3.805</v>
+      </c>
+      <c r="H78">
+        <v>3.773</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79">
-        <v>230012</v>
+        <v>230526</v>
       </c>
       <c r="C79" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D79">
-        <v>3.914</v>
+        <v>3.935</v>
       </c>
       <c r="E79">
-        <v>3.778</v>
+        <v>3.947</v>
       </c>
       <c r="F79">
-        <v>3.595</v>
+        <v>3.495</v>
       </c>
       <c r="G79">
-        <v>3.737</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7">
+        <v>3.714</v>
+      </c>
+      <c r="H79">
+        <v>3.772</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
       <c r="A80">
         <v>79</v>
       </c>
       <c r="B80">
-        <v>230017</v>
+        <v>230016</v>
       </c>
       <c r="C80" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D80">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="E80">
-        <v>3.947</v>
+        <v>3.911</v>
       </c>
       <c r="F80">
-        <v>3.441</v>
+        <v>3.479</v>
       </c>
       <c r="G80">
-        <v>3.737</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7">
+        <v>3.691</v>
+      </c>
+      <c r="H80">
+        <v>3.77</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
       <c r="A81">
         <v>80</v>
       </c>
       <c r="B81">
-        <v>230473</v>
+        <v>230375</v>
       </c>
       <c r="C81" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D81">
-        <v>3.892</v>
+        <v>3.85</v>
       </c>
       <c r="E81">
-        <v>3.908</v>
+        <v>3.686</v>
       </c>
       <c r="F81">
-        <v>3.443</v>
+        <v>3.599</v>
       </c>
       <c r="G81">
-        <v>3.726</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H81">
+        <v>3.767</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
       <c r="A82">
         <v>81</v>
       </c>
       <c r="B82">
-        <v>230407</v>
+        <v>230727</v>
       </c>
       <c r="C82" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D82">
-        <v>4</v>
+        <v>3.785</v>
       </c>
       <c r="E82">
-        <v>3.756</v>
+        <v>3.888</v>
       </c>
       <c r="F82">
-        <v>3.508</v>
+        <v>3.54</v>
       </c>
       <c r="G82">
-        <v>3.718</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7">
+        <v>3.85</v>
+      </c>
+      <c r="H82">
+        <v>3.765</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
       <c r="A83">
         <v>82</v>
       </c>
       <c r="B83">
-        <v>230147</v>
+        <v>230527</v>
       </c>
       <c r="C83" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D83">
-        <v>3.892</v>
+        <v>4</v>
       </c>
       <c r="E83">
-        <v>3.817</v>
+        <v>3.83</v>
       </c>
       <c r="F83">
-        <v>3.508</v>
+        <v>3.339</v>
       </c>
       <c r="G83">
-        <v>3.716</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7">
+        <v>3.873</v>
+      </c>
+      <c r="H83">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
       <c r="A84">
         <v>83</v>
       </c>
       <c r="B84">
-        <v>230077</v>
+        <v>230012</v>
       </c>
       <c r="C84" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D84">
-        <v>3.785</v>
+        <v>3.914</v>
       </c>
       <c r="E84">
-        <v>3.733</v>
+        <v>3.778</v>
       </c>
       <c r="F84">
-        <v>3.619</v>
+        <v>3.595</v>
       </c>
       <c r="G84">
-        <v>3.706</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7">
+        <v>3.742</v>
+      </c>
+      <c r="H84">
+        <v>3.757</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
       <c r="A85">
         <v>84</v>
       </c>
       <c r="B85">
-        <v>230495</v>
+        <v>230065</v>
       </c>
       <c r="C85" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D85">
-        <v>3.85</v>
+        <v>3.892</v>
       </c>
       <c r="E85">
-        <v>3.869</v>
+        <v>3.83</v>
       </c>
       <c r="F85">
-        <v>3.443</v>
+        <v>3.347</v>
       </c>
       <c r="G85">
-        <v>3.701</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H85">
+        <v>3.751</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
       <c r="A86">
         <v>85</v>
       </c>
       <c r="B86">
-        <v>230444</v>
+        <v>230613</v>
       </c>
       <c r="C86" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D86">
-        <v>3.785</v>
+        <v>4</v>
       </c>
       <c r="E86">
-        <v>3.596</v>
+        <v>3.947</v>
       </c>
       <c r="F86">
-        <v>3.757</v>
+        <v>3.699</v>
       </c>
       <c r="G86">
-        <v>3.693</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7">
+        <v>3.357</v>
+      </c>
+      <c r="H86">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
       <c r="A87">
         <v>86</v>
       </c>
       <c r="B87">
-        <v>230261</v>
+        <v>230327</v>
       </c>
       <c r="C87" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D87">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E87">
-        <v>3.747</v>
+        <v>3.656</v>
       </c>
       <c r="F87">
-        <v>3.458</v>
+        <v>3.765</v>
       </c>
       <c r="G87">
-        <v>3.691</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7">
+        <v>3.705</v>
+      </c>
+      <c r="H87">
+        <v>3.744</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
       <c r="A88">
         <v>87</v>
       </c>
       <c r="B88">
-        <v>230375</v>
+        <v>230077</v>
       </c>
       <c r="C88" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D88">
-        <v>3.85</v>
+        <v>3.785</v>
       </c>
       <c r="E88">
-        <v>3.686</v>
+        <v>3.733</v>
       </c>
       <c r="F88">
-        <v>3.599</v>
+        <v>3.619</v>
       </c>
       <c r="G88">
-        <v>3.691</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7">
+        <v>3.824</v>
+      </c>
+      <c r="H88">
+        <v>3.74</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
       <c r="A89">
         <v>88</v>
       </c>
       <c r="B89">
-        <v>230527</v>
+        <v>230495</v>
       </c>
       <c r="C89" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D89">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E89">
-        <v>3.83</v>
+        <v>3.869</v>
       </c>
       <c r="F89">
-        <v>3.339</v>
+        <v>3.443</v>
       </c>
       <c r="G89">
-        <v>3.681</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7">
+        <v>3.766</v>
+      </c>
+      <c r="H89">
+        <v>3.732</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
       <c r="A90">
         <v>89</v>
       </c>
       <c r="B90">
-        <v>230013</v>
+        <v>230444</v>
       </c>
       <c r="C90" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D90">
-        <v>3.85</v>
+        <v>3.785</v>
       </c>
       <c r="E90">
-        <v>3.617</v>
+        <v>3.596</v>
       </c>
       <c r="F90">
-        <v>3.638</v>
+        <v>3.757</v>
       </c>
       <c r="G90">
-        <v>3.677</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7">
+        <v>3.75</v>
+      </c>
+      <c r="H90">
+        <v>3.722</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
       <c r="A91">
         <v>90</v>
       </c>
       <c r="B91">
-        <v>230458</v>
+        <v>230052</v>
       </c>
       <c r="C91" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D91">
-        <v>3.957</v>
+        <v>3.75</v>
       </c>
       <c r="E91">
-        <v>3.713</v>
+        <v>3.844</v>
       </c>
       <c r="F91">
-        <v>3.465</v>
+        <v>3.63</v>
       </c>
       <c r="G91">
-        <v>3.675</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7">
+        <v>3.65</v>
+      </c>
+      <c r="H91">
+        <v>3.718</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
       <c r="A92">
         <v>91</v>
       </c>
       <c r="B92">
-        <v>230229</v>
+        <v>230395</v>
       </c>
       <c r="C92" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D92">
         <v>3.85</v>
       </c>
       <c r="E92">
-        <v>3.817</v>
+        <v>3.656</v>
       </c>
       <c r="F92">
-        <v>3.4</v>
+        <v>3.334</v>
       </c>
       <c r="G92">
-        <v>3.674</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7">
+        <v>3.936</v>
+      </c>
+      <c r="H92">
+        <v>3.694</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8">
       <c r="A93">
         <v>92</v>
       </c>
       <c r="B93">
-        <v>230735</v>
+        <v>230563</v>
       </c>
       <c r="C93" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D93">
-        <v>3.935</v>
+        <v>3.892</v>
       </c>
       <c r="E93">
-        <v>3.786</v>
+        <v>3.726</v>
       </c>
       <c r="F93">
-        <v>3.399</v>
+        <v>3.304</v>
       </c>
       <c r="G93">
-        <v>3.673</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7">
+        <v>3.852</v>
+      </c>
+      <c r="H93">
+        <v>3.693</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
       <c r="A94">
         <v>93</v>
       </c>
       <c r="B94">
-        <v>230248</v>
+        <v>230650</v>
       </c>
       <c r="C94" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D94">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E94">
-        <v>3.634</v>
+        <v>3.708</v>
       </c>
       <c r="F94">
-        <v>3.543</v>
+        <v>3.373</v>
       </c>
       <c r="G94">
-        <v>3.67</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7">
+        <v>3.678</v>
+      </c>
+      <c r="H94">
+        <v>3.689</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
       <c r="A95">
         <v>94</v>
       </c>
       <c r="B95">
-        <v>230065</v>
+        <v>230458</v>
       </c>
       <c r="C95" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D95">
-        <v>3.892</v>
+        <v>3.957</v>
       </c>
       <c r="E95">
-        <v>3.83</v>
+        <v>3.713</v>
       </c>
       <c r="F95">
-        <v>3.347</v>
+        <v>3.465</v>
       </c>
       <c r="G95">
-        <v>3.659</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7">
+        <v>3.615</v>
+      </c>
+      <c r="H95">
+        <v>3.687</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
       <c r="A96">
         <v>95</v>
       </c>
       <c r="B96">
-        <v>230650</v>
+        <v>230229</v>
       </c>
       <c r="C96" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D96">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E96">
-        <v>3.708</v>
+        <v>3.817</v>
       </c>
       <c r="F96">
-        <v>3.373</v>
+        <v>3.4</v>
       </c>
       <c r="G96">
-        <v>3.648</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7">
+        <v>3.631</v>
+      </c>
+      <c r="H96">
+        <v>3.674</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
       <c r="A97">
         <v>96</v>
       </c>
       <c r="B97">
-        <v>230208</v>
+        <v>230013</v>
       </c>
       <c r="C97" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D97">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E97">
         <v>3.617</v>
       </c>
       <c r="F97">
-        <v>3.46</v>
+        <v>3.638</v>
       </c>
       <c r="G97">
-        <v>3.646</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7">
+        <v>3.578</v>
+      </c>
+      <c r="H97">
+        <v>3.67</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2953,7 +3247,7 @@
         <v>230175</v>
       </c>
       <c r="C98" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D98">
         <v>3.957</v>
@@ -2965,421 +3259,478 @@
         <v>3.404</v>
       </c>
       <c r="G98">
-        <v>3.645</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7">
+        <v>3.576</v>
+      </c>
+      <c r="H98">
+        <v>3.658</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8">
       <c r="A99">
         <v>98</v>
       </c>
       <c r="B99">
-        <v>230520</v>
+        <v>230208</v>
       </c>
       <c r="C99" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D99">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E99">
-        <v>3.726</v>
+        <v>3.617</v>
       </c>
       <c r="F99">
-        <v>3.43</v>
+        <v>3.46</v>
       </c>
       <c r="G99">
-        <v>3.641</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7">
+        <v>3.547</v>
+      </c>
+      <c r="H99">
+        <v>3.656</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8">
       <c r="A100">
         <v>99</v>
       </c>
       <c r="B100">
-        <v>230563</v>
+        <v>230280</v>
       </c>
       <c r="C100" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D100">
-        <v>3.892</v>
+        <v>3.85</v>
       </c>
       <c r="E100">
-        <v>3.726</v>
+        <v>3.908</v>
       </c>
       <c r="F100">
-        <v>3.304</v>
+        <v>3.13</v>
       </c>
       <c r="G100">
-        <v>3.603</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7">
+        <v>3.676</v>
+      </c>
+      <c r="H100">
+        <v>3.641</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8">
       <c r="A101">
         <v>100</v>
       </c>
       <c r="B101">
-        <v>230280</v>
+        <v>230520</v>
       </c>
       <c r="C101" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D101">
         <v>3.85</v>
       </c>
       <c r="E101">
-        <v>3.908</v>
+        <v>3.726</v>
       </c>
       <c r="F101">
-        <v>3.13</v>
+        <v>3.43</v>
       </c>
       <c r="G101">
-        <v>3.596</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7">
+        <v>3.513</v>
+      </c>
+      <c r="H101">
+        <v>3.629</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8">
       <c r="A102">
         <v>101</v>
       </c>
       <c r="B102">
-        <v>230259</v>
+        <v>230033</v>
       </c>
       <c r="C102" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D102">
         <v>3.85</v>
       </c>
       <c r="E102">
-        <v>3.551</v>
+        <v>3.604</v>
       </c>
       <c r="F102">
-        <v>3.447</v>
+        <v>3.347</v>
       </c>
       <c r="G102">
-        <v>3.583</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7">
+        <v>3.676</v>
+      </c>
+      <c r="H102">
+        <v>3.619</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8">
       <c r="A103">
         <v>102</v>
       </c>
       <c r="B103">
-        <v>230395</v>
+        <v>230564</v>
       </c>
       <c r="C103" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D103">
-        <v>3.85</v>
+        <v>3.871</v>
       </c>
       <c r="E103">
-        <v>3.656</v>
+        <v>3.421</v>
       </c>
       <c r="F103">
-        <v>3.334</v>
+        <v>3.221</v>
       </c>
       <c r="G103">
-        <v>3.578</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7">
+        <v>3.914</v>
+      </c>
+      <c r="H103">
+        <v>3.606</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8">
       <c r="A104">
         <v>103</v>
       </c>
       <c r="B104">
-        <v>230020</v>
+        <v>230636</v>
       </c>
       <c r="C104" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D104">
-        <v>4</v>
+        <v>3.892</v>
       </c>
       <c r="E104">
-        <v>3.856</v>
+        <v>3.578</v>
       </c>
       <c r="F104">
-        <v>3.004</v>
+        <v>3.278</v>
       </c>
       <c r="G104">
-        <v>3.563</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7">
+        <v>3.676</v>
+      </c>
+      <c r="H104">
+        <v>3.606</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8">
       <c r="A105">
         <v>104</v>
       </c>
       <c r="B105">
-        <v>230033</v>
+        <v>230493</v>
       </c>
       <c r="C105" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D105">
-        <v>3.85</v>
+        <v>3.935</v>
       </c>
       <c r="E105">
-        <v>3.604</v>
+        <v>3.46</v>
       </c>
       <c r="F105">
-        <v>3.347</v>
+        <v>3.334</v>
       </c>
       <c r="G105">
-        <v>3.563</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7">
+        <v>3.678</v>
+      </c>
+      <c r="H105">
+        <v>3.601</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8">
       <c r="A106">
         <v>105</v>
       </c>
       <c r="B106">
-        <v>230636</v>
+        <v>230581</v>
       </c>
       <c r="C106" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D106">
-        <v>3.892</v>
+        <v>3.792</v>
       </c>
       <c r="E106">
-        <v>3.578</v>
+        <v>3.629</v>
       </c>
       <c r="F106">
-        <v>3.278</v>
+        <v>3.014</v>
       </c>
       <c r="G106">
-        <v>3.536</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7">
+        <v>3.9</v>
+      </c>
+      <c r="H106">
+        <v>3.583</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8">
       <c r="A107">
         <v>106</v>
       </c>
       <c r="B107">
-        <v>230224</v>
+        <v>230020</v>
       </c>
       <c r="C107" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D107">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E107">
-        <v>3.486</v>
+        <v>3.856</v>
       </c>
       <c r="F107">
-        <v>3.221</v>
+        <v>3.004</v>
       </c>
       <c r="G107">
-        <v>3.47</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7">
+        <v>3.336</v>
+      </c>
+      <c r="H107">
+        <v>3.549</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8">
       <c r="A108">
         <v>107</v>
       </c>
       <c r="B108">
-        <v>230581</v>
+        <v>230248</v>
       </c>
       <c r="C108" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D108">
-        <v>3.792</v>
+        <v>3.935</v>
       </c>
       <c r="E108">
-        <v>3.629</v>
+        <v>3.634</v>
       </c>
       <c r="F108">
-        <v>3.014</v>
+        <v>3.543</v>
       </c>
       <c r="G108">
-        <v>3.465</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7">
+        <v>2.933</v>
+      </c>
+      <c r="H108">
+        <v>3.511</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8">
       <c r="A109">
         <v>108</v>
       </c>
       <c r="B109">
-        <v>230268</v>
+        <v>230224</v>
       </c>
       <c r="C109" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D109">
         <v>3.85</v>
       </c>
       <c r="E109">
-        <v>3.586</v>
+        <v>3.486</v>
       </c>
       <c r="F109">
-        <v>3.095</v>
+        <v>3.221</v>
       </c>
       <c r="G109">
-        <v>3.46</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7">
+        <v>3.468</v>
+      </c>
+      <c r="H109">
+        <v>3.506</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8">
       <c r="A110">
         <v>109</v>
       </c>
       <c r="B110">
-        <v>230564</v>
+        <v>230259</v>
       </c>
       <c r="C110" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D110">
-        <v>3.871</v>
+        <v>3.85</v>
       </c>
       <c r="E110">
-        <v>3.421</v>
+        <v>3.551</v>
       </c>
       <c r="F110">
-        <v>3.221</v>
+        <v>3.447</v>
       </c>
       <c r="G110">
-        <v>3.45</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7">
+        <v>3.099</v>
+      </c>
+      <c r="H110">
+        <v>3.486</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8">
       <c r="A111">
         <v>110</v>
       </c>
       <c r="B111">
-        <v>230238</v>
+        <v>230268</v>
       </c>
       <c r="C111" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D111">
-        <v>3.764</v>
+        <v>3.85</v>
       </c>
       <c r="E111">
-        <v>3.459</v>
+        <v>3.586</v>
       </c>
       <c r="F111">
-        <v>3.214</v>
+        <v>3.095</v>
       </c>
       <c r="G111">
-        <v>3.445</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7">
+        <v>2.99</v>
+      </c>
+      <c r="H111">
+        <v>3.38</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8">
       <c r="A112">
         <v>111</v>
       </c>
       <c r="B112">
-        <v>230493</v>
+        <v>230449</v>
       </c>
       <c r="C112" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D112">
-        <v>3.935</v>
+        <v>3.807</v>
       </c>
       <c r="E112">
-        <v>3.069</v>
+        <v>3.266</v>
       </c>
       <c r="F112">
-        <v>3.334</v>
+        <v>2.835</v>
       </c>
       <c r="G112">
-        <v>3.373</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7">
+        <v>3.416</v>
+      </c>
+      <c r="H112">
+        <v>3.331</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8">
       <c r="A113">
         <v>112</v>
       </c>
       <c r="B113">
-        <v>230203</v>
+        <v>230238</v>
       </c>
       <c r="C113" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D113">
-        <v>3.85</v>
+        <v>3.764</v>
       </c>
       <c r="E113">
-        <v>3.456</v>
+        <v>3.459</v>
       </c>
       <c r="F113">
-        <v>2.785</v>
+        <v>3.214</v>
       </c>
       <c r="G113">
-        <v>3.308</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7">
+        <v>2.591</v>
+      </c>
+      <c r="H113">
+        <v>3.256</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8">
       <c r="A114">
         <v>113</v>
       </c>
       <c r="B114">
-        <v>230449</v>
+        <v>230730</v>
       </c>
       <c r="C114" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D114">
-        <v>3.807</v>
+        <v>4</v>
       </c>
       <c r="E114">
-        <v>3.266</v>
+        <v>3.626</v>
       </c>
       <c r="F114">
-        <v>2.835</v>
+        <v>2.343</v>
       </c>
       <c r="G114">
-        <v>3.249</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7">
+        <v>3.019</v>
+      </c>
+      <c r="H114">
+        <v>3.247</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8">
       <c r="A115">
         <v>114</v>
       </c>
       <c r="B115">
-        <v>230730</v>
+        <v>230183</v>
       </c>
       <c r="C115" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D115">
         <v>4</v>
       </c>
       <c r="E115">
-        <v>3.626</v>
+        <v>3.508</v>
       </c>
       <c r="F115">
-        <v>2.343</v>
+        <v>2.404</v>
       </c>
       <c r="G115">
-        <v>3.221</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7">
+        <v>2.852</v>
+      </c>
+      <c r="H115">
+        <v>3.191</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8">
       <c r="A116">
         <v>115</v>
       </c>
       <c r="B116">
-        <v>230183</v>
+        <v>230203</v>
       </c>
       <c r="C116" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D116">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E116">
-        <v>3.508</v>
+        <v>3.456</v>
       </c>
       <c r="F116">
-        <v>2.404</v>
+        <v>2.785</v>
       </c>
       <c r="G116">
-        <v>3.2</v>
+        <v>1.484</v>
+      </c>
+      <c r="H116">
+        <v>2.893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
With EDR and CGPA fixed
</commit_message>
<xml_diff>
--- a/output/CGPA_Results.xlsx
+++ b/output/CGPA_Results.xlsx
@@ -64,252 +64,252 @@
     <t>PERERA W.A.L.S.</t>
   </si>
   <si>
+    <t>KUMARA K.B.R.</t>
+  </si>
+  <si>
     <t>RATHNAYAKE M.A.G.K.N.</t>
   </si>
   <si>
+    <t>BANDARA H.Y.W.</t>
+  </si>
+  <si>
+    <t>PERERA K.W.A.O.V.</t>
+  </si>
+  <si>
+    <t>WANIGASUNDARA W.M.H.</t>
+  </si>
+  <si>
+    <t>KUMARASINGHE M.N.</t>
+  </si>
+  <si>
+    <t>PERERA U.I.H.</t>
+  </si>
+  <si>
+    <t>COLOMBAGE D.M.</t>
+  </si>
+  <si>
+    <t>IMADUWAGE O.N.H.</t>
+  </si>
+  <si>
+    <t>FERNANDO W.H.D.</t>
+  </si>
+  <si>
+    <t>ILANKOON I.M.M.K.B.</t>
+  </si>
+  <si>
+    <t>KARIYAWASAM J.H.D.</t>
+  </si>
+  <si>
+    <t>SAMARASINGHE S.M.R.R.</t>
+  </si>
+  <si>
+    <t>DE MEL D.J.</t>
+  </si>
+  <si>
+    <t>GARUSINGHE S.B.</t>
+  </si>
+  <si>
+    <t>ARACHCHI A.D.I.D.</t>
+  </si>
+  <si>
+    <t>DISSANAYAKA D.M.D.P.</t>
+  </si>
+  <si>
+    <t>KEERAWELLA K.P.C.P.</t>
+  </si>
+  <si>
+    <t>BANDARA W.D.A.C.</t>
+  </si>
+  <si>
     <t>DISSANAYAKE G.R.G.K.</t>
   </si>
   <si>
-    <t>PERERA U.I.H.</t>
-  </si>
-  <si>
-    <t>KUMARASINGHE M.N.</t>
-  </si>
-  <si>
-    <t>WANIGASUNDARA W.M.H.</t>
-  </si>
-  <si>
-    <t>BANDARA H.Y.W.</t>
-  </si>
-  <si>
-    <t>KUMARA K.B.R.</t>
-  </si>
-  <si>
-    <t>ILANKOON I.M.M.K.B.</t>
-  </si>
-  <si>
-    <t>KARIYAWASAM J.H.D.</t>
-  </si>
-  <si>
-    <t>IMADUWAGE O.N.H.</t>
-  </si>
-  <si>
-    <t>PERERA K.W.A.O.V.</t>
-  </si>
-  <si>
-    <t>SAMARASINGHE S.M.R.R.</t>
-  </si>
-  <si>
-    <t>GARUSINGHE S.B.</t>
-  </si>
-  <si>
-    <t>ARACHCHI A.D.I.D.</t>
+    <t>KARUNARATHNA G.K.T.</t>
+  </si>
+  <si>
+    <t>RANASINGHE D.P.H.</t>
+  </si>
+  <si>
+    <t>RAHUL B.</t>
   </si>
   <si>
     <t>MALDENIYA P.A.D.G.R.</t>
   </si>
   <si>
-    <t>DISSANAYAKA D.M.D.P.</t>
-  </si>
-  <si>
-    <t>COLOMBAGE D.M.</t>
-  </si>
-  <si>
-    <t>DE MEL D.J.</t>
-  </si>
-  <si>
-    <t>FERNANDO W.H.D.</t>
-  </si>
-  <si>
-    <t>KARUNARATHNA G.K.T.</t>
-  </si>
-  <si>
     <t>PEIRIS E.A.S.S.</t>
   </si>
   <si>
-    <t>BANDARA W.D.A.C.</t>
-  </si>
-  <si>
-    <t>RANASINGHE D.P.H.</t>
-  </si>
-  <si>
-    <t>KEERAWELLA K.P.C.P.</t>
-  </si>
-  <si>
-    <t>RAHUL B.</t>
+    <t>WEDAMESTRIGE A.N.</t>
+  </si>
+  <si>
+    <t>ANTHONY C.S.B.</t>
   </si>
   <si>
     <t>CHANDRAKUMARA H.A.D.C.</t>
   </si>
   <si>
-    <t>WEDAMESTRIGE A.N.</t>
+    <t>GUNASEKARA L.U.A.</t>
   </si>
   <si>
     <t>AMARATHUNGE A.M.N.L.</t>
   </si>
   <si>
-    <t>GUNASEKARA L.U.A.</t>
+    <t>RASANJANA W.P.G.R.A.</t>
   </si>
   <si>
     <t>WIJESEKARA W.A.G.S.</t>
   </si>
   <si>
+    <t>GUNATHUNGA U.A.</t>
+  </si>
+  <si>
     <t>RATHEESHAN A.R.</t>
   </si>
   <si>
-    <t>RASANJANA W.P.G.R.A.</t>
-  </si>
-  <si>
-    <t>GUNATHUNGA U.A.</t>
+    <t>JAYAWEERA N.S.</t>
+  </si>
+  <si>
+    <t>MUNASINGHE A.I.</t>
   </si>
   <si>
     <t>DESHAN W.U.</t>
   </si>
   <si>
-    <t>ANTHONY C.S.B.</t>
-  </si>
-  <si>
-    <t>MUNASINGHE A.I.</t>
+    <t>UPEKSHANI T.S.</t>
   </si>
   <si>
     <t>PEIRIS T.S.R.</t>
   </si>
   <si>
-    <t>JAYAWEERA N.S.</t>
+    <t>WEERAKOON A.H.T.M.</t>
+  </si>
+  <si>
+    <t>KUMARA P.K.M.P.</t>
+  </si>
+  <si>
+    <t>PATHIRANA P.T.S.</t>
+  </si>
+  <si>
+    <t>PITIWADUGE D.N.</t>
+  </si>
+  <si>
+    <t>PRIYADARSHANA S.A.D.</t>
+  </si>
+  <si>
+    <t>DILHAN W.A.</t>
   </si>
   <si>
     <t>DHARMAKEERTHI P.K.G.C.L.</t>
   </si>
   <si>
-    <t>WEERAKOON A.H.T.M.</t>
-  </si>
-  <si>
-    <t>KUMARA P.K.M.P.</t>
-  </si>
-  <si>
-    <t>PRIYADARSHANA S.A.D.</t>
-  </si>
-  <si>
-    <t>UPEKSHANI T.S.</t>
-  </si>
-  <si>
-    <t>DILHAN W.A.</t>
-  </si>
-  <si>
-    <t>PITIWADUGE D.N.</t>
-  </si>
-  <si>
-    <t>PATHIRANA P.T.S.</t>
+    <t>FERNANDO H.M.D.</t>
   </si>
   <si>
     <t>KARUNANAYAKE A.H.D.</t>
   </si>
   <si>
-    <t>FERNANDO H.M.D.</t>
+    <t>RAHMAN M.F.A.</t>
+  </si>
+  <si>
+    <t>TENNAKOON U.G.R.B.</t>
+  </si>
+  <si>
+    <t>AROSHANA H.A.P.</t>
+  </si>
+  <si>
+    <t>GAMAGE SK</t>
   </si>
   <si>
     <t>PRISHMIKA H.W.N.</t>
   </si>
   <si>
-    <t>TENNAKOON U.G.R.B.</t>
-  </si>
-  <si>
-    <t>AROSHANA H.A.P.</t>
-  </si>
-  <si>
-    <t>GAMAGE SK</t>
-  </si>
-  <si>
     <t>PERERA H.A.J.I.</t>
   </si>
   <si>
     <t>GUNASEKARA K.S.</t>
   </si>
   <si>
-    <t>RAHMAN M.F.A.</t>
-  </si>
-  <si>
     <t>BALASOORIYA B.R.B.D.</t>
   </si>
   <si>
+    <t>WEERASINGHE J.A.H.R.</t>
+  </si>
+  <si>
+    <t>WIJESINGHE U.G.S.K.D.</t>
+  </si>
+  <si>
+    <t>RANATHUNGA R.J.K.O.H.</t>
+  </si>
+  <si>
+    <t>WIJESINGHE W.A.P.W.</t>
+  </si>
+  <si>
+    <t>ATHUKORALA U.R.</t>
+  </si>
+  <si>
+    <t>DILHARA D.S.</t>
+  </si>
+  <si>
     <t>UMAIR A.</t>
   </si>
   <si>
-    <t>RANATHUNGA R.J.K.O.H.</t>
-  </si>
-  <si>
-    <t>WEERASINGHE J.A.H.R.</t>
-  </si>
-  <si>
-    <t>WIJESINGHE U.G.S.K.D.</t>
+    <t>DISSANAYAKE R.K.T.</t>
   </si>
   <si>
     <t>MEEDENIYA M.M.H.</t>
   </si>
   <si>
+    <t>ABISHEK L.</t>
+  </si>
+  <si>
+    <t>RANAWAKA R.A.C.D.</t>
+  </si>
+  <si>
+    <t>SARUKA U.</t>
+  </si>
+  <si>
+    <t>WITHANAGE G.D.N.</t>
+  </si>
+  <si>
+    <t>INDUWARA M.L.A.S.</t>
+  </si>
+  <si>
+    <t>LENMINI B.L.W.</t>
+  </si>
+  <si>
     <t>PERAMUNAGE D.S.</t>
   </si>
   <si>
-    <t>ATHUKORALA U.R.</t>
-  </si>
-  <si>
-    <t>DILHARA D.S.</t>
-  </si>
-  <si>
-    <t>INDUWARA M.L.A.S.</t>
-  </si>
-  <si>
-    <t>WITHANAGE G.D.N.</t>
-  </si>
-  <si>
-    <t>DISSANAYAKE R.K.T.</t>
-  </si>
-  <si>
-    <t>SARUKA U.</t>
+    <t>ARACHCHIGE M. A. D. T. S.</t>
+  </si>
+  <si>
+    <t>SHEHAN M.N.N.</t>
   </si>
   <si>
     <t>ADHIKARI A.H.C.S.</t>
   </si>
   <si>
-    <t>RANAWAKA R.A.C.D.</t>
-  </si>
-  <si>
-    <t>ABISHEK L.</t>
-  </si>
-  <si>
-    <t>LENMINI B.L.W.</t>
-  </si>
-  <si>
-    <t>WIJESINGHE W.A.P.W.</t>
+    <t>KAUSHALYA R.G.S.P.</t>
+  </si>
+  <si>
+    <t>ABEYWARDHANA T.C.W.</t>
+  </si>
+  <si>
+    <t>AYANAJA N.B.G.M.</t>
+  </si>
+  <si>
+    <t>BANDARA K.M.N.D.</t>
+  </si>
+  <si>
+    <t>NIRMANI W.T.</t>
   </si>
   <si>
     <t>RANAWAKA R.A.G.K.</t>
   </si>
   <si>
-    <t>ABEYWARDHANA T.C.W.</t>
-  </si>
-  <si>
-    <t>AYANAJA N.B.G.M.</t>
-  </si>
-  <si>
-    <t>SHEHAN M.N.N.</t>
-  </si>
-  <si>
-    <t>KAUSHALYA R.G.S.P.</t>
-  </si>
-  <si>
-    <t>BANDARA K.M.N.D.</t>
-  </si>
-  <si>
     <t>PRABHARSHA H.W.D.</t>
   </si>
   <si>
-    <t>NIRMANI W.T.</t>
-  </si>
-  <si>
-    <t>ARACHCHIGE M. A. D. T. S.</t>
-  </si>
-  <si>
     <t>MANATUNGA K.D.</t>
   </si>
   <si>
@@ -319,42 +319,45 @@
     <t>UBEYSEKARA V.T.T.</t>
   </si>
   <si>
+    <t>ABEYWARNA D.H.</t>
+  </si>
+  <si>
+    <t>HANSINDU M.M.A.D.</t>
+  </si>
+  <si>
     <t>PALIHENA H.H.</t>
   </si>
   <si>
-    <t>HANSINDU M.M.A.D.</t>
-  </si>
-  <si>
-    <t>ABEYWARNA D.H.</t>
-  </si>
-  <si>
     <t>ERANGA W.A.O.</t>
   </si>
   <si>
+    <t>JAYASINGHE J.A.P.R.</t>
+  </si>
+  <si>
     <t>GUNASEKARA H.M.</t>
   </si>
   <si>
-    <t>JAYASINGHE J.A.P.R.</t>
+    <t>AMARASINGHE A.A.D.K.</t>
+  </si>
+  <si>
+    <t>THARUSHIKA G.K.E.</t>
   </si>
   <si>
     <t>RANASINGHE A.G.N.S.</t>
   </si>
   <si>
-    <t>AMARASINGHE A.A.D.K.</t>
+    <t>PIYUMAL N.P.P.</t>
   </si>
   <si>
     <t>SAMARASEKARA S.M.R.P.</t>
   </si>
   <si>
-    <t>THARUSHIKA G.K.E.</t>
-  </si>
-  <si>
-    <t>PIYUMAL N.P.P.</t>
-  </si>
-  <si>
     <t>SANTHOSH S.</t>
   </si>
   <si>
+    <t>IMBULPITIYA B.N.</t>
+  </si>
+  <si>
     <t>AHAMED A.M.S.</t>
   </si>
   <si>
@@ -364,16 +367,13 @@
     <t>HAKAM M.R.A.</t>
   </si>
   <si>
-    <t>IMBULPITIYA B.N.</t>
+    <t>HENDENIYA H.M.J.C.</t>
   </si>
   <si>
     <t>JAYAKODY J.A.C.P.</t>
   </si>
   <si>
     <t>NUWANAKA W.A.S.</t>
-  </si>
-  <si>
-    <t>HENDENIYA H.M.J.C.</t>
   </si>
   <si>
     <t>WIJETHILAKA J.S.</t>
@@ -792,7 +792,7 @@
         <v>4</v>
       </c>
       <c r="H3">
-        <v>3.993</v>
+        <v>3.992</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -818,7 +818,7 @@
         <v>4</v>
       </c>
       <c r="H4">
-        <v>3.993</v>
+        <v>3.992</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -844,7 +844,7 @@
         <v>4</v>
       </c>
       <c r="H5">
-        <v>3.99</v>
+        <v>3.989</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -870,7 +870,7 @@
         <v>4</v>
       </c>
       <c r="H6">
-        <v>3.99</v>
+        <v>3.989</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -896,7 +896,7 @@
         <v>4</v>
       </c>
       <c r="H7">
-        <v>3.99</v>
+        <v>3.989</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -922,7 +922,7 @@
         <v>4</v>
       </c>
       <c r="H8">
-        <v>3.989</v>
+        <v>3.988</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -945,10 +945,10 @@
         <v>4</v>
       </c>
       <c r="G9">
-        <v>3.936</v>
+        <v>3.945</v>
       </c>
       <c r="H9">
-        <v>3.984</v>
+        <v>3.985</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -956,25 +956,25 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>230544</v>
+        <v>230352</v>
       </c>
       <c r="C10" t="s">
         <v>16</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E10">
         <v>4</v>
       </c>
       <c r="F10">
-        <v>3.921</v>
+        <v>3.96</v>
       </c>
       <c r="G10">
         <v>4</v>
       </c>
       <c r="H10">
-        <v>3.98</v>
+        <v>3.978</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -982,7 +982,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>230159</v>
+        <v>230544</v>
       </c>
       <c r="C11" t="s">
         <v>17</v>
@@ -991,16 +991,16 @@
         <v>4</v>
       </c>
       <c r="E11">
-        <v>3.955</v>
+        <v>4</v>
       </c>
       <c r="F11">
-        <v>3.954</v>
+        <v>3.921</v>
       </c>
       <c r="G11">
         <v>4</v>
       </c>
       <c r="H11">
-        <v>3.977</v>
+        <v>3.978</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1008,7 +1008,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>230486</v>
+        <v>230074</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
@@ -1020,13 +1020,13 @@
         <v>4</v>
       </c>
       <c r="F12">
-        <v>3.907</v>
+        <v>3.96</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>3.945</v>
       </c>
       <c r="H12">
-        <v>3.976</v>
+        <v>3.974</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1034,25 +1034,25 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>230355</v>
+        <v>230481</v>
       </c>
       <c r="C13" t="s">
         <v>19</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E13">
         <v>4</v>
       </c>
       <c r="F13">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="G13">
         <v>4</v>
       </c>
       <c r="H13">
-        <v>3.975</v>
+        <v>3.974</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1078,7 +1078,7 @@
         <v>4</v>
       </c>
       <c r="H14">
-        <v>3.975</v>
+        <v>3.973</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1086,7 +1086,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>230074</v>
+        <v>230355</v>
       </c>
       <c r="C15" t="s">
         <v>21</v>
@@ -1098,13 +1098,13 @@
         <v>4</v>
       </c>
       <c r="F15">
-        <v>3.96</v>
+        <v>3.9</v>
       </c>
       <c r="G15">
-        <v>3.936</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>3.974</v>
+        <v>3.971</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1112,25 +1112,25 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>230352</v>
+        <v>230486</v>
       </c>
       <c r="C16" t="s">
         <v>22</v>
       </c>
       <c r="D16">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E16">
         <v>4</v>
       </c>
       <c r="F16">
-        <v>3.96</v>
+        <v>3.907</v>
       </c>
       <c r="G16">
         <v>4</v>
       </c>
       <c r="H16">
-        <v>3.973</v>
+        <v>3.971</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1138,25 +1138,25 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>230256</v>
+        <v>230108</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
       </c>
       <c r="D17">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E17">
         <v>4</v>
       </c>
       <c r="F17">
-        <v>3.925</v>
+        <v>3.954</v>
       </c>
       <c r="G17">
-        <v>3.936</v>
+        <v>3.959</v>
       </c>
       <c r="H17">
-        <v>3.965</v>
+        <v>3.967</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1164,25 +1164,25 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>230318</v>
+        <v>230258</v>
       </c>
       <c r="C18" t="s">
         <v>24</v>
       </c>
       <c r="D18">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E18">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F18">
-        <v>3.924</v>
+        <v>3.957</v>
       </c>
       <c r="G18">
-        <v>3.936</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>3.965</v>
+        <v>3.966</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1190,25 +1190,25 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>230258</v>
+        <v>230186</v>
       </c>
       <c r="C19" t="s">
         <v>25</v>
       </c>
       <c r="D19">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E19">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F19">
-        <v>3.957</v>
+        <v>3.869</v>
       </c>
       <c r="G19">
         <v>4</v>
       </c>
       <c r="H19">
-        <v>3.963</v>
+        <v>3.964</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1216,25 +1216,25 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>230481</v>
+        <v>230256</v>
       </c>
       <c r="C20" t="s">
         <v>26</v>
       </c>
       <c r="D20">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E20">
         <v>4</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>3.925</v>
       </c>
       <c r="G20">
-        <v>4</v>
+        <v>3.945</v>
       </c>
       <c r="H20">
-        <v>3.962</v>
+        <v>3.963</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1242,25 +1242,25 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>230566</v>
+        <v>230318</v>
       </c>
       <c r="C21" t="s">
         <v>27</v>
       </c>
       <c r="D21">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E21">
         <v>4</v>
       </c>
       <c r="F21">
-        <v>3.884</v>
+        <v>3.924</v>
       </c>
       <c r="G21">
-        <v>4</v>
+        <v>3.945</v>
       </c>
       <c r="H21">
-        <v>3.96</v>
+        <v>3.963</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1268,25 +1268,25 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>230197</v>
+        <v>230566</v>
       </c>
       <c r="C22" t="s">
         <v>28</v>
       </c>
       <c r="D22">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E22">
-        <v>3.934</v>
+        <v>4</v>
       </c>
       <c r="F22">
-        <v>3.899</v>
+        <v>3.884</v>
       </c>
       <c r="G22">
         <v>4</v>
       </c>
       <c r="H22">
-        <v>3.958</v>
+        <v>3.957</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1294,25 +1294,25 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>230051</v>
+        <v>230121</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E23">
         <v>4</v>
       </c>
       <c r="F23">
-        <v>3.83</v>
+        <v>3.921</v>
       </c>
       <c r="G23">
-        <v>4</v>
+        <v>3.945</v>
       </c>
       <c r="H23">
-        <v>3.957</v>
+        <v>3.956</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1320,7 +1320,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>230390</v>
+        <v>230197</v>
       </c>
       <c r="C24" t="s">
         <v>30</v>
@@ -1329,16 +1329,16 @@
         <v>4</v>
       </c>
       <c r="E24">
-        <v>4</v>
+        <v>3.934</v>
       </c>
       <c r="F24">
-        <v>3.873</v>
+        <v>3.899</v>
       </c>
       <c r="G24">
-        <v>3.952</v>
+        <v>4</v>
       </c>
       <c r="H24">
-        <v>3.956</v>
+        <v>3.954</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1346,7 +1346,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>230155</v>
+        <v>230051</v>
       </c>
       <c r="C25" t="s">
         <v>31</v>
@@ -1355,16 +1355,16 @@
         <v>4</v>
       </c>
       <c r="E25">
-        <v>3.921</v>
+        <v>4</v>
       </c>
       <c r="F25">
-        <v>3.957</v>
+        <v>3.83</v>
       </c>
       <c r="G25">
-        <v>3.942</v>
+        <v>4</v>
       </c>
       <c r="H25">
-        <v>3.955</v>
+        <v>3.952</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1372,25 +1372,25 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>230108</v>
+        <v>230155</v>
       </c>
       <c r="C26" t="s">
         <v>32</v>
       </c>
       <c r="D26">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E26">
-        <v>4</v>
+        <v>3.921</v>
       </c>
       <c r="F26">
-        <v>3.954</v>
+        <v>3.957</v>
       </c>
       <c r="G26">
-        <v>3.925</v>
+        <v>3.949</v>
       </c>
       <c r="H26">
-        <v>3.953</v>
+        <v>3.952</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1398,25 +1398,25 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>230121</v>
+        <v>230332</v>
       </c>
       <c r="C27" t="s">
         <v>33</v>
       </c>
       <c r="D27">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E27">
         <v>4</v>
       </c>
       <c r="F27">
-        <v>3.921</v>
+        <v>3.79</v>
       </c>
       <c r="G27">
-        <v>3.936</v>
+        <v>4</v>
       </c>
       <c r="H27">
-        <v>3.953</v>
+        <v>3.951</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1424,7 +1424,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>230186</v>
+        <v>230082</v>
       </c>
       <c r="C28" t="s">
         <v>34</v>
@@ -1436,13 +1436,13 @@
         <v>4</v>
       </c>
       <c r="F28">
-        <v>3.869</v>
+        <v>3.96</v>
       </c>
       <c r="G28">
-        <v>3.942</v>
+        <v>3.862</v>
       </c>
       <c r="H28">
-        <v>3.952</v>
+        <v>3.95</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1450,7 +1450,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>230322</v>
+        <v>230159</v>
       </c>
       <c r="C29" t="s">
         <v>35</v>
@@ -1459,16 +1459,16 @@
         <v>4</v>
       </c>
       <c r="E29">
-        <v>3.908</v>
+        <v>3.955</v>
       </c>
       <c r="F29">
-        <v>3.9</v>
+        <v>3.954</v>
       </c>
       <c r="G29">
-        <v>4</v>
+        <v>3.904</v>
       </c>
       <c r="H29">
-        <v>3.952</v>
+        <v>3.949</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1476,7 +1476,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>230469</v>
+        <v>230322</v>
       </c>
       <c r="C30" t="s">
         <v>36</v>
@@ -1485,16 +1485,16 @@
         <v>4</v>
       </c>
       <c r="E30">
-        <v>3.96</v>
+        <v>3.908</v>
       </c>
       <c r="F30">
-        <v>3.937</v>
+        <v>3.9</v>
       </c>
       <c r="G30">
-        <v>3.914</v>
+        <v>4</v>
       </c>
       <c r="H30">
-        <v>3.952</v>
+        <v>3.947</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1502,7 +1502,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>230082</v>
+        <v>230521</v>
       </c>
       <c r="C31" t="s">
         <v>37</v>
@@ -1514,13 +1514,13 @@
         <v>4</v>
       </c>
       <c r="F31">
-        <v>3.96</v>
+        <v>3.843</v>
       </c>
       <c r="G31">
-        <v>3.842</v>
+        <v>3.964</v>
       </c>
       <c r="H31">
-        <v>3.95</v>
+        <v>3.947</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1528,7 +1528,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>230521</v>
+        <v>230508</v>
       </c>
       <c r="C32" t="s">
         <v>38</v>
@@ -1540,13 +1540,13 @@
         <v>4</v>
       </c>
       <c r="F32">
-        <v>3.843</v>
+        <v>3.882</v>
       </c>
       <c r="G32">
-        <v>3.959</v>
+        <v>3.872</v>
       </c>
       <c r="H32">
-        <v>3.95</v>
+        <v>3.932</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1554,7 +1554,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>230332</v>
+        <v>230390</v>
       </c>
       <c r="C33" t="s">
         <v>39</v>
@@ -1566,13 +1566,13 @@
         <v>4</v>
       </c>
       <c r="F33">
-        <v>3.79</v>
+        <v>3.873</v>
       </c>
       <c r="G33">
-        <v>4</v>
+        <v>3.863</v>
       </c>
       <c r="H33">
-        <v>3.947</v>
+        <v>3.928</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1580,7 +1580,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>230508</v>
+        <v>230469</v>
       </c>
       <c r="C34" t="s">
         <v>40</v>
@@ -1589,16 +1589,16 @@
         <v>4</v>
       </c>
       <c r="E34">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F34">
-        <v>3.882</v>
+        <v>3.937</v>
       </c>
       <c r="G34">
-        <v>3.852</v>
+        <v>3.837</v>
       </c>
       <c r="H34">
-        <v>3.933</v>
+        <v>3.925</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1606,7 +1606,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>230100</v>
+        <v>230687</v>
       </c>
       <c r="C35" t="s">
         <v>41</v>
@@ -1615,16 +1615,16 @@
         <v>4</v>
       </c>
       <c r="E35">
-        <v>4</v>
+        <v>3.934</v>
       </c>
       <c r="F35">
-        <v>3.721</v>
+        <v>3.83</v>
       </c>
       <c r="G35">
-        <v>3.936</v>
+        <v>3.891</v>
       </c>
       <c r="H35">
-        <v>3.914</v>
+        <v>3.904</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1632,7 +1632,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>230687</v>
+        <v>230045</v>
       </c>
       <c r="C36" t="s">
         <v>42</v>
@@ -1641,16 +1641,16 @@
         <v>4</v>
       </c>
       <c r="E36">
-        <v>3.934</v>
+        <v>4</v>
       </c>
       <c r="F36">
-        <v>3.83</v>
+        <v>3.704</v>
       </c>
       <c r="G36">
-        <v>3.876</v>
+        <v>3.945</v>
       </c>
       <c r="H36">
-        <v>3.909</v>
+        <v>3.902</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1658,7 +1658,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>230038</v>
+        <v>230100</v>
       </c>
       <c r="C37" t="s">
         <v>43</v>
@@ -1670,13 +1670,13 @@
         <v>4</v>
       </c>
       <c r="F37">
-        <v>3.691</v>
+        <v>3.721</v>
       </c>
       <c r="G37">
-        <v>3.914</v>
+        <v>3.904</v>
       </c>
       <c r="H37">
-        <v>3.901</v>
+        <v>3.896</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1699,10 +1699,10 @@
         <v>3.821</v>
       </c>
       <c r="G38">
-        <v>3.936</v>
+        <v>3.945</v>
       </c>
       <c r="H38">
-        <v>3.899</v>
+        <v>3.895</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -1710,7 +1710,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>230724</v>
+        <v>230038</v>
       </c>
       <c r="C39" t="s">
         <v>45</v>
@@ -1719,16 +1719,16 @@
         <v>4</v>
       </c>
       <c r="E39">
-        <v>3.869</v>
+        <v>4</v>
       </c>
       <c r="F39">
-        <v>3.847</v>
+        <v>3.691</v>
       </c>
       <c r="G39">
-        <v>3.873</v>
+        <v>3.925</v>
       </c>
       <c r="H39">
-        <v>3.897</v>
+        <v>3.894</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -1736,25 +1736,25 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>230539</v>
+        <v>230536</v>
       </c>
       <c r="C40" t="s">
         <v>46</v>
       </c>
       <c r="D40">
-        <v>3.935</v>
+        <v>3.957</v>
       </c>
       <c r="E40">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F40">
-        <v>3.652</v>
+        <v>3.847</v>
       </c>
       <c r="G40">
-        <v>4</v>
+        <v>3.833</v>
       </c>
       <c r="H40">
-        <v>3.896</v>
+        <v>3.892</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -1762,25 +1762,25 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>230536</v>
+        <v>230724</v>
       </c>
       <c r="C41" t="s">
         <v>47</v>
       </c>
       <c r="D41">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E41">
-        <v>3.96</v>
+        <v>3.869</v>
       </c>
       <c r="F41">
         <v>3.847</v>
       </c>
       <c r="G41">
-        <v>3.809</v>
+        <v>3.89</v>
       </c>
       <c r="H41">
-        <v>3.893</v>
+        <v>3.891</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -1806,7 +1806,7 @@
         <v>4</v>
       </c>
       <c r="H42">
-        <v>3.892</v>
+        <v>3.885</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -1814,25 +1814,25 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>230130</v>
+        <v>230539</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
       </c>
       <c r="D43">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E43">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F43">
-        <v>3.714</v>
+        <v>3.652</v>
       </c>
       <c r="G43">
-        <v>3.889</v>
+        <v>3.964</v>
       </c>
       <c r="H43">
-        <v>3.89</v>
+        <v>3.884</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -1840,25 +1840,25 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>230045</v>
+        <v>230300</v>
       </c>
       <c r="C44" t="s">
         <v>50</v>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E44">
         <v>4</v>
       </c>
       <c r="F44">
-        <v>3.704</v>
+        <v>3.713</v>
       </c>
       <c r="G44">
-        <v>3.852</v>
+        <v>3.89</v>
       </c>
       <c r="H44">
-        <v>3.889</v>
+        <v>3.879</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -1881,10 +1881,10 @@
         <v>3.804</v>
       </c>
       <c r="G45">
-        <v>3.789</v>
+        <v>3.818</v>
       </c>
       <c r="H45">
-        <v>3.883</v>
+        <v>3.879</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -1892,7 +1892,7 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>230470</v>
+        <v>230130</v>
       </c>
       <c r="C46" t="s">
         <v>52</v>
@@ -1901,16 +1901,16 @@
         <v>4</v>
       </c>
       <c r="E46">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F46">
-        <v>3.526</v>
+        <v>3.714</v>
       </c>
       <c r="G46">
-        <v>4</v>
+        <v>3.863</v>
       </c>
       <c r="H46">
-        <v>3.881</v>
+        <v>3.876</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -1918,25 +1918,25 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>230300</v>
+        <v>230659</v>
       </c>
       <c r="C47" t="s">
         <v>53</v>
       </c>
       <c r="D47">
-        <v>3.935</v>
+        <v>3.857</v>
       </c>
       <c r="E47">
-        <v>4</v>
+        <v>3.869</v>
       </c>
       <c r="F47">
-        <v>3.713</v>
+        <v>3.804</v>
       </c>
       <c r="G47">
-        <v>3.873</v>
+        <v>3.945</v>
       </c>
       <c r="H47">
-        <v>3.88</v>
+        <v>3.869</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -1944,25 +1944,25 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>230140</v>
+        <v>230470</v>
       </c>
       <c r="C48" t="s">
         <v>54</v>
       </c>
       <c r="D48">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E48">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F48">
-        <v>3.873</v>
+        <v>3.526</v>
       </c>
       <c r="G48">
-        <v>3.742</v>
+        <v>4</v>
       </c>
       <c r="H48">
-        <v>3.877</v>
+        <v>3.867</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -1985,10 +1985,10 @@
         <v>3.771</v>
       </c>
       <c r="G49">
-        <v>3.709</v>
+        <v>3.745</v>
       </c>
       <c r="H49">
-        <v>3.87</v>
+        <v>3.867</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2014,7 +2014,7 @@
         <v>4</v>
       </c>
       <c r="H50">
-        <v>3.868</v>
+        <v>3.863</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2022,25 +2022,25 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>230502</v>
+        <v>230468</v>
       </c>
       <c r="C51" t="s">
         <v>57</v>
       </c>
       <c r="D51">
-        <v>4</v>
+        <v>3.914</v>
       </c>
       <c r="E51">
-        <v>3.947</v>
+        <v>4</v>
       </c>
       <c r="F51">
-        <v>3.586</v>
+        <v>3.895</v>
       </c>
       <c r="G51">
-        <v>3.936</v>
+        <v>3.65</v>
       </c>
       <c r="H51">
-        <v>3.867</v>
+        <v>3.862</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2048,25 +2048,25 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>230659</v>
+        <v>230492</v>
       </c>
       <c r="C52" t="s">
         <v>58</v>
       </c>
       <c r="D52">
-        <v>3.857</v>
+        <v>3.935</v>
       </c>
       <c r="E52">
-        <v>3.869</v>
+        <v>3.908</v>
       </c>
       <c r="F52">
-        <v>3.804</v>
+        <v>3.69</v>
       </c>
       <c r="G52">
-        <v>3.936</v>
+        <v>3.925</v>
       </c>
       <c r="H52">
-        <v>3.866</v>
+        <v>3.862</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2074,25 +2074,25 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>230145</v>
+        <v>230502</v>
       </c>
       <c r="C53" t="s">
         <v>59</v>
       </c>
       <c r="D53">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E53">
-        <v>4</v>
+        <v>3.947</v>
       </c>
       <c r="F53">
-        <v>3.704</v>
+        <v>3.586</v>
       </c>
       <c r="G53">
-        <v>3.809</v>
+        <v>3.945</v>
       </c>
       <c r="H53">
-        <v>3.862</v>
+        <v>3.854</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2100,7 +2100,7 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>230492</v>
+        <v>230145</v>
       </c>
       <c r="C54" t="s">
         <v>60</v>
@@ -2109,16 +2109,16 @@
         <v>3.935</v>
       </c>
       <c r="E54">
-        <v>3.908</v>
+        <v>4</v>
       </c>
       <c r="F54">
-        <v>3.69</v>
+        <v>3.704</v>
       </c>
       <c r="G54">
-        <v>3.914</v>
+        <v>3.796</v>
       </c>
       <c r="H54">
-        <v>3.861</v>
+        <v>3.849</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2126,25 +2126,25 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>230468</v>
+        <v>230140</v>
       </c>
       <c r="C55" t="s">
         <v>61</v>
       </c>
       <c r="D55">
-        <v>3.914</v>
+        <v>3.935</v>
       </c>
       <c r="E55">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F55">
-        <v>3.895</v>
+        <v>3.873</v>
       </c>
       <c r="G55">
-        <v>3.594</v>
+        <v>3.64</v>
       </c>
       <c r="H55">
-        <v>3.85</v>
+        <v>3.846</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2152,25 +2152,25 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>230321</v>
+        <v>230180</v>
       </c>
       <c r="C56" t="s">
         <v>62</v>
       </c>
       <c r="D56">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E56">
-        <v>3.947</v>
+        <v>3.817</v>
       </c>
       <c r="F56">
-        <v>3.73</v>
+        <v>3.778</v>
       </c>
       <c r="G56">
-        <v>3.704</v>
+        <v>3.862</v>
       </c>
       <c r="H56">
-        <v>3.845</v>
+        <v>3.839</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2178,25 +2178,25 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>230180</v>
+        <v>230321</v>
       </c>
       <c r="C57" t="s">
         <v>63</v>
       </c>
       <c r="D57">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E57">
-        <v>3.817</v>
+        <v>3.947</v>
       </c>
       <c r="F57">
-        <v>3.778</v>
+        <v>3.73</v>
       </c>
       <c r="G57">
-        <v>3.842</v>
+        <v>3.741</v>
       </c>
       <c r="H57">
-        <v>3.843</v>
+        <v>3.838</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2204,25 +2204,25 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>230500</v>
+        <v>230507</v>
       </c>
       <c r="C58" t="s">
         <v>64</v>
       </c>
       <c r="D58">
-        <v>3.957</v>
+        <v>3.857</v>
       </c>
       <c r="E58">
-        <v>3.908</v>
+        <v>3.877</v>
       </c>
       <c r="F58">
-        <v>3.678</v>
+        <v>3.645</v>
       </c>
       <c r="G58">
-        <v>3.826</v>
+        <v>3.945</v>
       </c>
       <c r="H58">
-        <v>3.842</v>
+        <v>3.836</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2245,10 +2245,10 @@
         <v>3.726</v>
       </c>
       <c r="G59">
-        <v>3.771</v>
+        <v>3.8</v>
       </c>
       <c r="H59">
-        <v>3.84</v>
+        <v>3.835</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2271,10 +2271,10 @@
         <v>3.713</v>
       </c>
       <c r="G60">
-        <v>3.726</v>
+        <v>3.763</v>
       </c>
       <c r="H60">
-        <v>3.836</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2297,10 +2297,10 @@
         <v>3.678</v>
       </c>
       <c r="G61">
-        <v>3.914</v>
+        <v>3.925</v>
       </c>
       <c r="H61">
-        <v>3.834</v>
+        <v>3.826</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2308,25 +2308,25 @@
         <v>61</v>
       </c>
       <c r="B62">
-        <v>230477</v>
+        <v>230500</v>
       </c>
       <c r="C62" t="s">
         <v>68</v>
       </c>
       <c r="D62">
-        <v>3.935</v>
+        <v>3.957</v>
       </c>
       <c r="E62">
-        <v>3.817</v>
+        <v>3.908</v>
       </c>
       <c r="F62">
-        <v>3.873</v>
+        <v>3.678</v>
       </c>
       <c r="G62">
-        <v>3.704</v>
+        <v>3.809</v>
       </c>
       <c r="H62">
-        <v>3.832</v>
+        <v>3.825</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2334,25 +2334,25 @@
         <v>62</v>
       </c>
       <c r="B63">
-        <v>230211</v>
+        <v>230477</v>
       </c>
       <c r="C63" t="s">
         <v>69</v>
       </c>
       <c r="D63">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E63">
-        <v>3.895</v>
+        <v>3.817</v>
       </c>
       <c r="F63">
-        <v>3.782</v>
+        <v>3.873</v>
       </c>
       <c r="G63">
-        <v>3.647</v>
+        <v>3.704</v>
       </c>
       <c r="H63">
-        <v>3.831</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2360,25 +2360,25 @@
         <v>63</v>
       </c>
       <c r="B64">
-        <v>230507</v>
+        <v>230211</v>
       </c>
       <c r="C64" t="s">
         <v>70</v>
       </c>
       <c r="D64">
-        <v>3.857</v>
+        <v>4</v>
       </c>
       <c r="E64">
-        <v>3.877</v>
+        <v>3.895</v>
       </c>
       <c r="F64">
-        <v>3.645</v>
+        <v>3.782</v>
       </c>
       <c r="G64">
-        <v>3.9</v>
+        <v>3.654</v>
       </c>
       <c r="H64">
-        <v>3.819</v>
+        <v>3.817</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -2401,10 +2401,10 @@
         <v>3.717</v>
       </c>
       <c r="G65">
-        <v>3.789</v>
+        <v>3.818</v>
       </c>
       <c r="H65">
-        <v>3.817</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -2412,25 +2412,25 @@
         <v>65</v>
       </c>
       <c r="B66">
-        <v>230654</v>
+        <v>230697</v>
       </c>
       <c r="C66" t="s">
         <v>72</v>
       </c>
       <c r="D66">
-        <v>3.935</v>
+        <v>3.957</v>
       </c>
       <c r="E66">
-        <v>3.839</v>
+        <v>3.96</v>
       </c>
       <c r="F66">
-        <v>3.591</v>
+        <v>3.671</v>
       </c>
       <c r="G66">
-        <v>3.871</v>
+        <v>3.679</v>
       </c>
       <c r="H66">
-        <v>3.809</v>
+        <v>3.803</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -2438,25 +2438,25 @@
         <v>66</v>
       </c>
       <c r="B67">
-        <v>230525</v>
+        <v>230726</v>
       </c>
       <c r="C67" t="s">
         <v>73</v>
       </c>
       <c r="D67">
-        <v>4</v>
+        <v>3.892</v>
       </c>
       <c r="E67">
-        <v>4</v>
+        <v>3.869</v>
       </c>
       <c r="F67">
-        <v>3.5</v>
+        <v>3.66</v>
       </c>
       <c r="G67">
-        <v>3.726</v>
+        <v>3.818</v>
       </c>
       <c r="H67">
-        <v>3.806</v>
+        <v>3.801</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -2464,25 +2464,25 @@
         <v>67</v>
       </c>
       <c r="B68">
-        <v>230697</v>
+        <v>230525</v>
       </c>
       <c r="C68" t="s">
         <v>74</v>
       </c>
       <c r="D68">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E68">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F68">
-        <v>3.671</v>
+        <v>3.5</v>
       </c>
       <c r="G68">
-        <v>3.633</v>
+        <v>3.763</v>
       </c>
       <c r="H68">
-        <v>3.805</v>
+        <v>3.796</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -2490,25 +2490,25 @@
         <v>68</v>
       </c>
       <c r="B69">
-        <v>230726</v>
+        <v>230727</v>
       </c>
       <c r="C69" t="s">
         <v>75</v>
       </c>
       <c r="D69">
-        <v>3.892</v>
+        <v>3.785</v>
       </c>
       <c r="E69">
-        <v>3.869</v>
+        <v>3.888</v>
       </c>
       <c r="F69">
-        <v>3.66</v>
+        <v>3.54</v>
       </c>
       <c r="G69">
-        <v>3.789</v>
+        <v>3.918</v>
       </c>
       <c r="H69">
-        <v>3.802</v>
+        <v>3.795</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -2516,7 +2516,7 @@
         <v>69</v>
       </c>
       <c r="B70">
-        <v>230407</v>
+        <v>230063</v>
       </c>
       <c r="C70" t="s">
         <v>76</v>
@@ -2525,16 +2525,16 @@
         <v>4</v>
       </c>
       <c r="E70">
-        <v>3.756</v>
+        <v>3.908</v>
       </c>
       <c r="F70">
-        <v>3.508</v>
+        <v>3.56</v>
       </c>
       <c r="G70">
-        <v>3.936</v>
+        <v>3.745</v>
       </c>
       <c r="H70">
-        <v>3.8</v>
+        <v>3.782</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -2542,7 +2542,7 @@
         <v>70</v>
       </c>
       <c r="B71">
-        <v>230473</v>
+        <v>230147</v>
       </c>
       <c r="C71" t="s">
         <v>77</v>
@@ -2551,16 +2551,16 @@
         <v>3.892</v>
       </c>
       <c r="E71">
-        <v>3.908</v>
+        <v>3.817</v>
       </c>
       <c r="F71">
-        <v>3.443</v>
+        <v>3.508</v>
       </c>
       <c r="G71">
-        <v>3.936</v>
+        <v>3.945</v>
       </c>
       <c r="H71">
-        <v>3.794</v>
+        <v>3.778</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -2568,25 +2568,25 @@
         <v>71</v>
       </c>
       <c r="B72">
-        <v>230063</v>
+        <v>230654</v>
       </c>
       <c r="C72" t="s">
         <v>78</v>
       </c>
       <c r="D72">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E72">
-        <v>3.908</v>
+        <v>3.839</v>
       </c>
       <c r="F72">
-        <v>3.56</v>
+        <v>3.591</v>
       </c>
       <c r="G72">
-        <v>3.705</v>
+        <v>3.799</v>
       </c>
       <c r="H72">
-        <v>3.793</v>
+        <v>3.776</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -2594,25 +2594,25 @@
         <v>72</v>
       </c>
       <c r="B73">
-        <v>230147</v>
+        <v>230164</v>
       </c>
       <c r="C73" t="s">
         <v>79</v>
       </c>
       <c r="D73">
-        <v>3.892</v>
+        <v>3.957</v>
       </c>
       <c r="E73">
-        <v>3.817</v>
+        <v>3.869</v>
       </c>
       <c r="F73">
-        <v>3.508</v>
+        <v>3.626</v>
       </c>
       <c r="G73">
-        <v>3.936</v>
+        <v>3.708</v>
       </c>
       <c r="H73">
-        <v>3.788</v>
+        <v>3.771</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -2620,7 +2620,7 @@
         <v>73</v>
       </c>
       <c r="B74">
-        <v>230261</v>
+        <v>230407</v>
       </c>
       <c r="C74" t="s">
         <v>80</v>
@@ -2629,16 +2629,16 @@
         <v>4</v>
       </c>
       <c r="E74">
-        <v>3.747</v>
+        <v>3.756</v>
       </c>
       <c r="F74">
-        <v>3.458</v>
+        <v>3.508</v>
       </c>
       <c r="G74">
-        <v>3.936</v>
+        <v>3.904</v>
       </c>
       <c r="H74">
-        <v>3.785</v>
+        <v>3.768</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -2646,25 +2646,25 @@
         <v>74</v>
       </c>
       <c r="B75">
-        <v>230735</v>
+        <v>230016</v>
       </c>
       <c r="C75" t="s">
         <v>81</v>
       </c>
       <c r="D75">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E75">
-        <v>3.786</v>
+        <v>3.911</v>
       </c>
       <c r="F75">
-        <v>3.399</v>
+        <v>3.479</v>
       </c>
       <c r="G75">
-        <v>4</v>
+        <v>3.695</v>
       </c>
       <c r="H75">
-        <v>3.78</v>
+        <v>3.765</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -2672,25 +2672,25 @@
         <v>75</v>
       </c>
       <c r="B76">
-        <v>230164</v>
+        <v>230526</v>
       </c>
       <c r="C76" t="s">
         <v>82</v>
       </c>
       <c r="D76">
-        <v>3.957</v>
+        <v>3.935</v>
       </c>
       <c r="E76">
-        <v>3.869</v>
+        <v>3.947</v>
       </c>
       <c r="F76">
-        <v>3.626</v>
+        <v>3.495</v>
       </c>
       <c r="G76">
-        <v>3.666</v>
+        <v>3.75</v>
       </c>
       <c r="H76">
-        <v>3.779</v>
+        <v>3.765</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -2713,10 +2713,10 @@
         <v>3.543</v>
       </c>
       <c r="G77">
-        <v>3.676</v>
+        <v>3.679</v>
       </c>
       <c r="H77">
-        <v>3.778</v>
+        <v>3.761</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -2724,25 +2724,25 @@
         <v>77</v>
       </c>
       <c r="B78">
-        <v>230017</v>
+        <v>230735</v>
       </c>
       <c r="C78" t="s">
         <v>84</v>
       </c>
       <c r="D78">
-        <v>3.9</v>
+        <v>3.935</v>
       </c>
       <c r="E78">
-        <v>3.947</v>
+        <v>3.786</v>
       </c>
       <c r="F78">
-        <v>3.441</v>
+        <v>3.399</v>
       </c>
       <c r="G78">
-        <v>3.805</v>
+        <v>4</v>
       </c>
       <c r="H78">
-        <v>3.773</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -2750,25 +2750,25 @@
         <v>78</v>
       </c>
       <c r="B79">
-        <v>230526</v>
+        <v>230261</v>
       </c>
       <c r="C79" t="s">
         <v>85</v>
       </c>
       <c r="D79">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E79">
-        <v>3.947</v>
+        <v>3.747</v>
       </c>
       <c r="F79">
-        <v>3.495</v>
+        <v>3.458</v>
       </c>
       <c r="G79">
-        <v>3.714</v>
+        <v>3.945</v>
       </c>
       <c r="H79">
-        <v>3.772</v>
+        <v>3.759</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -2776,25 +2776,25 @@
         <v>79</v>
       </c>
       <c r="B80">
-        <v>230016</v>
+        <v>230375</v>
       </c>
       <c r="C80" t="s">
         <v>86</v>
       </c>
       <c r="D80">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E80">
-        <v>3.911</v>
+        <v>3.686</v>
       </c>
       <c r="F80">
-        <v>3.479</v>
+        <v>3.599</v>
       </c>
       <c r="G80">
-        <v>3.691</v>
+        <v>3.945</v>
       </c>
       <c r="H80">
-        <v>3.77</v>
+        <v>3.759</v>
       </c>
     </row>
     <row r="81" spans="1:8">
@@ -2802,25 +2802,25 @@
         <v>80</v>
       </c>
       <c r="B81">
-        <v>230375</v>
+        <v>230473</v>
       </c>
       <c r="C81" t="s">
         <v>87</v>
       </c>
       <c r="D81">
-        <v>3.85</v>
+        <v>3.892</v>
       </c>
       <c r="E81">
-        <v>3.686</v>
+        <v>3.908</v>
       </c>
       <c r="F81">
-        <v>3.599</v>
+        <v>3.443</v>
       </c>
       <c r="G81">
-        <v>3.936</v>
+        <v>3.849</v>
       </c>
       <c r="H81">
-        <v>3.767</v>
+        <v>3.759</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -2828,25 +2828,25 @@
         <v>81</v>
       </c>
       <c r="B82">
-        <v>230727</v>
+        <v>230052</v>
       </c>
       <c r="C82" t="s">
         <v>88</v>
       </c>
       <c r="D82">
-        <v>3.785</v>
+        <v>3.75</v>
       </c>
       <c r="E82">
-        <v>3.888</v>
+        <v>3.844</v>
       </c>
       <c r="F82">
-        <v>3.54</v>
+        <v>3.63</v>
       </c>
       <c r="G82">
-        <v>3.85</v>
+        <v>3.768</v>
       </c>
       <c r="H82">
-        <v>3.765</v>
+        <v>3.756</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -2854,7 +2854,7 @@
         <v>82</v>
       </c>
       <c r="B83">
-        <v>230527</v>
+        <v>230613</v>
       </c>
       <c r="C83" t="s">
         <v>89</v>
@@ -2863,16 +2863,16 @@
         <v>4</v>
       </c>
       <c r="E83">
-        <v>3.83</v>
+        <v>3.947</v>
       </c>
       <c r="F83">
-        <v>3.339</v>
+        <v>3.699</v>
       </c>
       <c r="G83">
-        <v>3.873</v>
+        <v>3.445</v>
       </c>
       <c r="H83">
-        <v>3.76</v>
+        <v>3.752</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -2880,25 +2880,25 @@
         <v>83</v>
       </c>
       <c r="B84">
-        <v>230012</v>
+        <v>230017</v>
       </c>
       <c r="C84" t="s">
         <v>90</v>
       </c>
       <c r="D84">
-        <v>3.914</v>
+        <v>3.9</v>
       </c>
       <c r="E84">
-        <v>3.778</v>
+        <v>3.947</v>
       </c>
       <c r="F84">
-        <v>3.595</v>
+        <v>3.441</v>
       </c>
       <c r="G84">
-        <v>3.742</v>
+        <v>3.79</v>
       </c>
       <c r="H84">
-        <v>3.757</v>
+        <v>3.751</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -2906,25 +2906,25 @@
         <v>84</v>
       </c>
       <c r="B85">
-        <v>230065</v>
+        <v>230327</v>
       </c>
       <c r="C85" t="s">
         <v>91</v>
       </c>
       <c r="D85">
-        <v>3.892</v>
+        <v>3.85</v>
       </c>
       <c r="E85">
-        <v>3.83</v>
+        <v>3.708</v>
       </c>
       <c r="F85">
-        <v>3.347</v>
+        <v>3.765</v>
       </c>
       <c r="G85">
-        <v>3.936</v>
+        <v>3.681</v>
       </c>
       <c r="H85">
-        <v>3.751</v>
+        <v>3.741</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -2932,25 +2932,25 @@
         <v>85</v>
       </c>
       <c r="B86">
-        <v>230613</v>
+        <v>230012</v>
       </c>
       <c r="C86" t="s">
         <v>92</v>
       </c>
       <c r="D86">
-        <v>4</v>
+        <v>3.914</v>
       </c>
       <c r="E86">
-        <v>3.947</v>
+        <v>3.778</v>
       </c>
       <c r="F86">
-        <v>3.699</v>
+        <v>3.595</v>
       </c>
       <c r="G86">
-        <v>3.357</v>
+        <v>3.736</v>
       </c>
       <c r="H86">
-        <v>3.75</v>
+        <v>3.737</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -2958,25 +2958,25 @@
         <v>86</v>
       </c>
       <c r="B87">
-        <v>230327</v>
+        <v>230065</v>
       </c>
       <c r="C87" t="s">
         <v>93</v>
       </c>
       <c r="D87">
-        <v>3.85</v>
+        <v>3.892</v>
       </c>
       <c r="E87">
-        <v>3.656</v>
+        <v>3.83</v>
       </c>
       <c r="F87">
-        <v>3.765</v>
+        <v>3.347</v>
       </c>
       <c r="G87">
-        <v>3.705</v>
+        <v>3.945</v>
       </c>
       <c r="H87">
-        <v>3.744</v>
+        <v>3.736</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -2999,10 +2999,10 @@
         <v>3.619</v>
       </c>
       <c r="G88">
-        <v>3.824</v>
+        <v>3.822</v>
       </c>
       <c r="H88">
-        <v>3.74</v>
+        <v>3.736</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -3010,25 +3010,25 @@
         <v>88</v>
       </c>
       <c r="B89">
-        <v>230495</v>
+        <v>230444</v>
       </c>
       <c r="C89" t="s">
         <v>95</v>
       </c>
       <c r="D89">
-        <v>3.85</v>
+        <v>3.785</v>
       </c>
       <c r="E89">
-        <v>3.869</v>
+        <v>3.596</v>
       </c>
       <c r="F89">
-        <v>3.443</v>
+        <v>3.757</v>
       </c>
       <c r="G89">
-        <v>3.766</v>
+        <v>3.822</v>
       </c>
       <c r="H89">
-        <v>3.732</v>
+        <v>3.727</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -3036,25 +3036,25 @@
         <v>89</v>
       </c>
       <c r="B90">
-        <v>230444</v>
+        <v>230527</v>
       </c>
       <c r="C90" t="s">
         <v>96</v>
       </c>
       <c r="D90">
-        <v>3.785</v>
+        <v>4</v>
       </c>
       <c r="E90">
-        <v>3.596</v>
+        <v>3.83</v>
       </c>
       <c r="F90">
-        <v>3.757</v>
+        <v>3.339</v>
       </c>
       <c r="G90">
-        <v>3.75</v>
+        <v>3.849</v>
       </c>
       <c r="H90">
-        <v>3.722</v>
+        <v>3.726</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -3062,25 +3062,25 @@
         <v>90</v>
       </c>
       <c r="B91">
-        <v>230052</v>
+        <v>230495</v>
       </c>
       <c r="C91" t="s">
         <v>97</v>
       </c>
       <c r="D91">
-        <v>3.75</v>
+        <v>3.85</v>
       </c>
       <c r="E91">
-        <v>3.844</v>
+        <v>3.869</v>
       </c>
       <c r="F91">
-        <v>3.63</v>
+        <v>3.443</v>
       </c>
       <c r="G91">
-        <v>3.65</v>
+        <v>3.758</v>
       </c>
       <c r="H91">
-        <v>3.718</v>
+        <v>3.717</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -3103,10 +3103,10 @@
         <v>3.334</v>
       </c>
       <c r="G92">
-        <v>3.936</v>
+        <v>3.945</v>
       </c>
       <c r="H92">
-        <v>3.694</v>
+        <v>3.676</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -3129,10 +3129,10 @@
         <v>3.304</v>
       </c>
       <c r="G93">
-        <v>3.852</v>
+        <v>3.872</v>
       </c>
       <c r="H93">
-        <v>3.693</v>
+        <v>3.675</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -3155,10 +3155,10 @@
         <v>3.373</v>
       </c>
       <c r="G94">
-        <v>3.678</v>
+        <v>3.722</v>
       </c>
       <c r="H94">
-        <v>3.689</v>
+        <v>3.668</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -3166,25 +3166,25 @@
         <v>94</v>
       </c>
       <c r="B95">
-        <v>230458</v>
+        <v>230013</v>
       </c>
       <c r="C95" t="s">
         <v>101</v>
       </c>
       <c r="D95">
-        <v>3.957</v>
+        <v>3.85</v>
       </c>
       <c r="E95">
-        <v>3.713</v>
+        <v>3.617</v>
       </c>
       <c r="F95">
-        <v>3.465</v>
+        <v>3.638</v>
       </c>
       <c r="G95">
-        <v>3.615</v>
+        <v>3.636</v>
       </c>
       <c r="H95">
-        <v>3.687</v>
+        <v>3.667</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -3207,10 +3207,10 @@
         <v>3.4</v>
       </c>
       <c r="G96">
-        <v>3.631</v>
+        <v>3.64</v>
       </c>
       <c r="H96">
-        <v>3.674</v>
+        <v>3.665</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -3218,25 +3218,25 @@
         <v>96</v>
       </c>
       <c r="B97">
-        <v>230013</v>
+        <v>230458</v>
       </c>
       <c r="C97" t="s">
         <v>103</v>
       </c>
       <c r="D97">
-        <v>3.85</v>
+        <v>3.957</v>
       </c>
       <c r="E97">
-        <v>3.617</v>
+        <v>3.713</v>
       </c>
       <c r="F97">
-        <v>3.638</v>
+        <v>3.465</v>
       </c>
       <c r="G97">
-        <v>3.578</v>
+        <v>3.627</v>
       </c>
       <c r="H97">
-        <v>3.67</v>
+        <v>3.662</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -3259,10 +3259,10 @@
         <v>3.404</v>
       </c>
       <c r="G98">
-        <v>3.576</v>
+        <v>3.629</v>
       </c>
       <c r="H98">
-        <v>3.658</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -3270,25 +3270,25 @@
         <v>98</v>
       </c>
       <c r="B99">
-        <v>230208</v>
+        <v>230280</v>
       </c>
       <c r="C99" t="s">
         <v>105</v>
       </c>
       <c r="D99">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E99">
-        <v>3.617</v>
+        <v>3.908</v>
       </c>
       <c r="F99">
-        <v>3.46</v>
+        <v>3.13</v>
       </c>
       <c r="G99">
-        <v>3.547</v>
+        <v>3.679</v>
       </c>
       <c r="H99">
-        <v>3.656</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="100" spans="1:8">
@@ -3296,25 +3296,25 @@
         <v>99</v>
       </c>
       <c r="B100">
-        <v>230280</v>
+        <v>230208</v>
       </c>
       <c r="C100" t="s">
         <v>106</v>
       </c>
       <c r="D100">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E100">
-        <v>3.908</v>
+        <v>3.617</v>
       </c>
       <c r="F100">
-        <v>3.13</v>
+        <v>3.46</v>
       </c>
       <c r="G100">
-        <v>3.676</v>
+        <v>3.513</v>
       </c>
       <c r="H100">
-        <v>3.641</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -3322,7 +3322,7 @@
         <v>100</v>
       </c>
       <c r="B101">
-        <v>230520</v>
+        <v>230033</v>
       </c>
       <c r="C101" t="s">
         <v>107</v>
@@ -3331,16 +3331,16 @@
         <v>3.85</v>
       </c>
       <c r="E101">
-        <v>3.726</v>
+        <v>3.604</v>
       </c>
       <c r="F101">
-        <v>3.43</v>
+        <v>3.347</v>
       </c>
       <c r="G101">
-        <v>3.513</v>
+        <v>3.716</v>
       </c>
       <c r="H101">
-        <v>3.629</v>
+        <v>3.607</v>
       </c>
     </row>
     <row r="102" spans="1:8">
@@ -3348,25 +3348,25 @@
         <v>101</v>
       </c>
       <c r="B102">
-        <v>230033</v>
+        <v>230636</v>
       </c>
       <c r="C102" t="s">
         <v>108</v>
       </c>
       <c r="D102">
-        <v>3.85</v>
+        <v>3.892</v>
       </c>
       <c r="E102">
-        <v>3.604</v>
+        <v>3.578</v>
       </c>
       <c r="F102">
-        <v>3.347</v>
+        <v>3.278</v>
       </c>
       <c r="G102">
-        <v>3.676</v>
+        <v>3.716</v>
       </c>
       <c r="H102">
-        <v>3.619</v>
+        <v>3.588</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -3374,25 +3374,25 @@
         <v>102</v>
       </c>
       <c r="B103">
-        <v>230564</v>
+        <v>230520</v>
       </c>
       <c r="C103" t="s">
         <v>109</v>
       </c>
       <c r="D103">
-        <v>3.871</v>
+        <v>3.85</v>
       </c>
       <c r="E103">
-        <v>3.421</v>
+        <v>3.726</v>
       </c>
       <c r="F103">
-        <v>3.221</v>
+        <v>3.43</v>
       </c>
       <c r="G103">
-        <v>3.914</v>
+        <v>3.452</v>
       </c>
       <c r="H103">
-        <v>3.606</v>
+        <v>3.585</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -3400,25 +3400,25 @@
         <v>103</v>
       </c>
       <c r="B104">
-        <v>230636</v>
+        <v>230493</v>
       </c>
       <c r="C104" t="s">
         <v>110</v>
       </c>
       <c r="D104">
-        <v>3.892</v>
+        <v>3.935</v>
       </c>
       <c r="E104">
-        <v>3.578</v>
+        <v>3.46</v>
       </c>
       <c r="F104">
-        <v>3.278</v>
+        <v>3.334</v>
       </c>
       <c r="G104">
-        <v>3.676</v>
+        <v>3.722</v>
       </c>
       <c r="H104">
-        <v>3.606</v>
+        <v>3.576</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -3426,25 +3426,25 @@
         <v>104</v>
       </c>
       <c r="B105">
-        <v>230493</v>
+        <v>230564</v>
       </c>
       <c r="C105" t="s">
         <v>111</v>
       </c>
       <c r="D105">
-        <v>3.935</v>
+        <v>3.871</v>
       </c>
       <c r="E105">
-        <v>3.46</v>
+        <v>3.421</v>
       </c>
       <c r="F105">
-        <v>3.334</v>
+        <v>3.221</v>
       </c>
       <c r="G105">
-        <v>3.678</v>
+        <v>3.837</v>
       </c>
       <c r="H105">
-        <v>3.601</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -3467,10 +3467,10 @@
         <v>3.014</v>
       </c>
       <c r="G106">
-        <v>3.9</v>
+        <v>3.809</v>
       </c>
       <c r="H106">
-        <v>3.583</v>
+        <v>3.556</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -3478,25 +3478,25 @@
         <v>106</v>
       </c>
       <c r="B107">
-        <v>230020</v>
+        <v>230259</v>
       </c>
       <c r="C107" t="s">
         <v>113</v>
       </c>
       <c r="D107">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E107">
-        <v>3.856</v>
+        <v>3.551</v>
       </c>
       <c r="F107">
-        <v>3.004</v>
+        <v>3.447</v>
       </c>
       <c r="G107">
-        <v>3.336</v>
+        <v>3.468</v>
       </c>
       <c r="H107">
-        <v>3.549</v>
+        <v>3.553</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -3504,25 +3504,25 @@
         <v>107</v>
       </c>
       <c r="B108">
-        <v>230248</v>
+        <v>230020</v>
       </c>
       <c r="C108" t="s">
         <v>114</v>
       </c>
       <c r="D108">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E108">
-        <v>3.634</v>
+        <v>3.856</v>
       </c>
       <c r="F108">
-        <v>3.543</v>
+        <v>3.004</v>
       </c>
       <c r="G108">
-        <v>2.933</v>
+        <v>3.427</v>
       </c>
       <c r="H108">
-        <v>3.511</v>
+        <v>3.526</v>
       </c>
     </row>
     <row r="109" spans="1:8">
@@ -3530,25 +3530,25 @@
         <v>108</v>
       </c>
       <c r="B109">
-        <v>230224</v>
+        <v>230248</v>
       </c>
       <c r="C109" t="s">
         <v>115</v>
       </c>
       <c r="D109">
-        <v>3.85</v>
+        <v>3.935</v>
       </c>
       <c r="E109">
+        <v>3.634</v>
+      </c>
+      <c r="F109">
+        <v>3.543</v>
+      </c>
+      <c r="G109">
+        <v>3.029</v>
+      </c>
+      <c r="H109">
         <v>3.486</v>
-      </c>
-      <c r="F109">
-        <v>3.221</v>
-      </c>
-      <c r="G109">
-        <v>3.468</v>
-      </c>
-      <c r="H109">
-        <v>3.506</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -3556,7 +3556,7 @@
         <v>109</v>
       </c>
       <c r="B110">
-        <v>230259</v>
+        <v>230224</v>
       </c>
       <c r="C110" t="s">
         <v>116</v>
@@ -3565,16 +3565,16 @@
         <v>3.85</v>
       </c>
       <c r="E110">
-        <v>3.551</v>
+        <v>3.486</v>
       </c>
       <c r="F110">
-        <v>3.447</v>
+        <v>3.221</v>
       </c>
       <c r="G110">
-        <v>3.099</v>
+        <v>3.404</v>
       </c>
       <c r="H110">
-        <v>3.486</v>
+        <v>3.452</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -3582,25 +3582,25 @@
         <v>110</v>
       </c>
       <c r="B111">
-        <v>230268</v>
+        <v>230238</v>
       </c>
       <c r="C111" t="s">
         <v>117</v>
       </c>
       <c r="D111">
-        <v>3.85</v>
+        <v>3.764</v>
       </c>
       <c r="E111">
-        <v>3.586</v>
+        <v>3.459</v>
       </c>
       <c r="F111">
-        <v>3.095</v>
+        <v>3.214</v>
       </c>
       <c r="G111">
-        <v>2.99</v>
+        <v>3.19</v>
       </c>
       <c r="H111">
-        <v>3.38</v>
+        <v>3.378</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -3608,25 +3608,25 @@
         <v>111</v>
       </c>
       <c r="B112">
-        <v>230449</v>
+        <v>230268</v>
       </c>
       <c r="C112" t="s">
         <v>118</v>
       </c>
       <c r="D112">
-        <v>3.807</v>
+        <v>3.85</v>
       </c>
       <c r="E112">
-        <v>3.266</v>
+        <v>3.586</v>
       </c>
       <c r="F112">
-        <v>2.835</v>
+        <v>3.095</v>
       </c>
       <c r="G112">
-        <v>3.416</v>
+        <v>2.954</v>
       </c>
       <c r="H112">
-        <v>3.331</v>
+        <v>3.315</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -3634,25 +3634,25 @@
         <v>112</v>
       </c>
       <c r="B113">
-        <v>230238</v>
+        <v>230449</v>
       </c>
       <c r="C113" t="s">
         <v>119</v>
       </c>
       <c r="D113">
-        <v>3.764</v>
+        <v>3.807</v>
       </c>
       <c r="E113">
-        <v>3.459</v>
+        <v>3.266</v>
       </c>
       <c r="F113">
-        <v>3.214</v>
+        <v>2.835</v>
       </c>
       <c r="G113">
-        <v>2.591</v>
+        <v>3.49</v>
       </c>
       <c r="H113">
-        <v>3.256</v>
+        <v>3.313</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -3675,10 +3675,10 @@
         <v>2.343</v>
       </c>
       <c r="G114">
-        <v>3.019</v>
+        <v>3.054</v>
       </c>
       <c r="H114">
-        <v>3.247</v>
+        <v>3.173</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -3701,10 +3701,10 @@
         <v>2.404</v>
       </c>
       <c r="G115">
-        <v>2.852</v>
+        <v>3.009</v>
       </c>
       <c r="H115">
-        <v>3.191</v>
+        <v>3.148</v>
       </c>
     </row>
     <row r="116" spans="1:8">
@@ -3727,10 +3727,10 @@
         <v>2.785</v>
       </c>
       <c r="G116">
-        <v>1.484</v>
+        <v>1.827</v>
       </c>
       <c r="H116">
-        <v>2.893</v>
+        <v>2.901</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Results after change of FCOD, ECD, Mechanics
</commit_message>
<xml_diff>
--- a/output/CGPA_Results.xlsx
+++ b/output/CGPA_Results.xlsx
@@ -85,6 +85,9 @@
     <t>PERERA U.I.H.</t>
   </si>
   <si>
+    <t>DE MEL D.J.</t>
+  </si>
+  <si>
     <t>COLOMBAGE D.M.</t>
   </si>
   <si>
@@ -103,9 +106,6 @@
     <t>SAMARASINGHE S.M.R.R.</t>
   </si>
   <si>
-    <t>DE MEL D.J.</t>
-  </si>
-  <si>
     <t>GARUSINGHE S.B.</t>
   </si>
   <si>
@@ -139,15 +139,15 @@
     <t>PEIRIS E.A.S.S.</t>
   </si>
   <si>
+    <t>CHANDRAKUMARA H.A.D.C.</t>
+  </si>
+  <si>
     <t>WEDAMESTRIGE A.N.</t>
   </si>
   <si>
     <t>ANTHONY C.S.B.</t>
   </si>
   <si>
-    <t>CHANDRAKUMARA H.A.D.C.</t>
-  </si>
-  <si>
     <t>GUNASEKARA L.U.A.</t>
   </si>
   <si>
@@ -244,6 +244,9 @@
     <t>WIJESINGHE W.A.P.W.</t>
   </si>
   <si>
+    <t>DISSANAYAKE R.K.T.</t>
+  </si>
+  <si>
     <t>ATHUKORALA U.R.</t>
   </si>
   <si>
@@ -253,9 +256,6 @@
     <t>UMAIR A.</t>
   </si>
   <si>
-    <t>DISSANAYAKE R.K.T.</t>
-  </si>
-  <si>
     <t>MEEDENIYA M.M.H.</t>
   </si>
   <si>
@@ -352,10 +352,10 @@
     <t>SAMARASEKARA S.M.R.P.</t>
   </si>
   <si>
+    <t>IMBULPITIYA B.N.</t>
+  </si>
+  <si>
     <t>SANTHOSH S.</t>
-  </si>
-  <si>
-    <t>IMBULPITIYA B.N.</t>
   </si>
   <si>
     <t>AHAMED A.M.S.</t>
@@ -1138,25 +1138,25 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>230108</v>
+        <v>230121</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
       </c>
       <c r="D17">
-        <v>3.935</v>
+        <v>3.957</v>
       </c>
       <c r="E17">
         <v>4</v>
       </c>
       <c r="F17">
-        <v>3.954</v>
+        <v>3.921</v>
       </c>
       <c r="G17">
-        <v>3.959</v>
+        <v>4</v>
       </c>
       <c r="H17">
-        <v>3.967</v>
+        <v>3.97</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1164,7 +1164,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>230258</v>
+        <v>230108</v>
       </c>
       <c r="C18" t="s">
         <v>24</v>
@@ -1173,16 +1173,16 @@
         <v>3.935</v>
       </c>
       <c r="E18">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F18">
-        <v>3.957</v>
+        <v>3.954</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>3.959</v>
       </c>
       <c r="H18">
-        <v>3.966</v>
+        <v>3.967</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1190,25 +1190,25 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>230186</v>
+        <v>230258</v>
       </c>
       <c r="C19" t="s">
         <v>25</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E19">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F19">
-        <v>3.869</v>
+        <v>3.957</v>
       </c>
       <c r="G19">
         <v>4</v>
       </c>
       <c r="H19">
-        <v>3.964</v>
+        <v>3.966</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1216,7 +1216,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>230256</v>
+        <v>230186</v>
       </c>
       <c r="C20" t="s">
         <v>26</v>
@@ -1228,13 +1228,13 @@
         <v>4</v>
       </c>
       <c r="F20">
-        <v>3.925</v>
+        <v>3.869</v>
       </c>
       <c r="G20">
-        <v>3.945</v>
+        <v>4</v>
       </c>
       <c r="H20">
-        <v>3.963</v>
+        <v>3.964</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1242,7 +1242,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>230318</v>
+        <v>230256</v>
       </c>
       <c r="C21" t="s">
         <v>27</v>
@@ -1254,7 +1254,7 @@
         <v>4</v>
       </c>
       <c r="F21">
-        <v>3.924</v>
+        <v>3.925</v>
       </c>
       <c r="G21">
         <v>3.945</v>
@@ -1268,25 +1268,25 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>230566</v>
+        <v>230318</v>
       </c>
       <c r="C22" t="s">
         <v>28</v>
       </c>
       <c r="D22">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E22">
         <v>4</v>
       </c>
       <c r="F22">
-        <v>3.884</v>
+        <v>3.924</v>
       </c>
       <c r="G22">
-        <v>4</v>
+        <v>3.945</v>
       </c>
       <c r="H22">
-        <v>3.957</v>
+        <v>3.963</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1294,7 +1294,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>230121</v>
+        <v>230566</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
@@ -1306,13 +1306,13 @@
         <v>4</v>
       </c>
       <c r="F23">
-        <v>3.921</v>
+        <v>3.884</v>
       </c>
       <c r="G23">
-        <v>3.945</v>
+        <v>4</v>
       </c>
       <c r="H23">
-        <v>3.956</v>
+        <v>3.957</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1606,7 +1606,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>230687</v>
+        <v>230100</v>
       </c>
       <c r="C35" t="s">
         <v>41</v>
@@ -1615,16 +1615,16 @@
         <v>4</v>
       </c>
       <c r="E35">
-        <v>3.934</v>
+        <v>4</v>
       </c>
       <c r="F35">
-        <v>3.83</v>
+        <v>3.721</v>
       </c>
       <c r="G35">
-        <v>3.891</v>
+        <v>3.959</v>
       </c>
       <c r="H35">
-        <v>3.904</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1632,7 +1632,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>230045</v>
+        <v>230687</v>
       </c>
       <c r="C36" t="s">
         <v>42</v>
@@ -1641,16 +1641,16 @@
         <v>4</v>
       </c>
       <c r="E36">
-        <v>4</v>
+        <v>3.934</v>
       </c>
       <c r="F36">
-        <v>3.704</v>
+        <v>3.83</v>
       </c>
       <c r="G36">
-        <v>3.945</v>
+        <v>3.891</v>
       </c>
       <c r="H36">
-        <v>3.902</v>
+        <v>3.904</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1658,7 +1658,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>230100</v>
+        <v>230045</v>
       </c>
       <c r="C37" t="s">
         <v>43</v>
@@ -1670,13 +1670,13 @@
         <v>4</v>
       </c>
       <c r="F37">
-        <v>3.721</v>
+        <v>3.704</v>
       </c>
       <c r="G37">
-        <v>3.904</v>
+        <v>3.945</v>
       </c>
       <c r="H37">
-        <v>3.896</v>
+        <v>3.902</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2516,25 +2516,25 @@
         <v>69</v>
       </c>
       <c r="B70">
-        <v>230063</v>
+        <v>230164</v>
       </c>
       <c r="C70" t="s">
         <v>76</v>
       </c>
       <c r="D70">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E70">
-        <v>3.908</v>
+        <v>3.869</v>
       </c>
       <c r="F70">
-        <v>3.56</v>
+        <v>3.626</v>
       </c>
       <c r="G70">
-        <v>3.745</v>
+        <v>3.775</v>
       </c>
       <c r="H70">
-        <v>3.782</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -2542,25 +2542,25 @@
         <v>70</v>
       </c>
       <c r="B71">
-        <v>230147</v>
+        <v>230063</v>
       </c>
       <c r="C71" t="s">
         <v>77</v>
       </c>
       <c r="D71">
-        <v>3.892</v>
+        <v>4</v>
       </c>
       <c r="E71">
-        <v>3.817</v>
+        <v>3.908</v>
       </c>
       <c r="F71">
-        <v>3.508</v>
+        <v>3.56</v>
       </c>
       <c r="G71">
-        <v>3.945</v>
+        <v>3.745</v>
       </c>
       <c r="H71">
-        <v>3.778</v>
+        <v>3.782</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -2568,25 +2568,25 @@
         <v>71</v>
       </c>
       <c r="B72">
-        <v>230654</v>
+        <v>230147</v>
       </c>
       <c r="C72" t="s">
         <v>78</v>
       </c>
       <c r="D72">
-        <v>3.935</v>
+        <v>3.892</v>
       </c>
       <c r="E72">
-        <v>3.839</v>
+        <v>3.817</v>
       </c>
       <c r="F72">
-        <v>3.591</v>
+        <v>3.508</v>
       </c>
       <c r="G72">
-        <v>3.799</v>
+        <v>3.945</v>
       </c>
       <c r="H72">
-        <v>3.776</v>
+        <v>3.778</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -2594,25 +2594,25 @@
         <v>72</v>
       </c>
       <c r="B73">
-        <v>230164</v>
+        <v>230654</v>
       </c>
       <c r="C73" t="s">
         <v>79</v>
       </c>
       <c r="D73">
-        <v>3.957</v>
+        <v>3.935</v>
       </c>
       <c r="E73">
-        <v>3.869</v>
+        <v>3.839</v>
       </c>
       <c r="F73">
-        <v>3.626</v>
+        <v>3.591</v>
       </c>
       <c r="G73">
-        <v>3.708</v>
+        <v>3.799</v>
       </c>
       <c r="H73">
-        <v>3.771</v>
+        <v>3.776</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -3452,25 +3452,25 @@
         <v>105</v>
       </c>
       <c r="B106">
-        <v>230581</v>
+        <v>230259</v>
       </c>
       <c r="C106" t="s">
         <v>112</v>
       </c>
       <c r="D106">
-        <v>3.792</v>
+        <v>3.85</v>
       </c>
       <c r="E106">
-        <v>3.629</v>
+        <v>3.551</v>
       </c>
       <c r="F106">
-        <v>3.014</v>
+        <v>3.447</v>
       </c>
       <c r="G106">
-        <v>3.809</v>
+        <v>3.468</v>
       </c>
       <c r="H106">
-        <v>3.556</v>
+        <v>3.553</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -3478,25 +3478,25 @@
         <v>106</v>
       </c>
       <c r="B107">
-        <v>230259</v>
+        <v>230581</v>
       </c>
       <c r="C107" t="s">
         <v>113</v>
       </c>
       <c r="D107">
-        <v>3.85</v>
+        <v>3.735</v>
       </c>
       <c r="E107">
-        <v>3.551</v>
+        <v>3.629</v>
       </c>
       <c r="F107">
-        <v>3.447</v>
+        <v>3.014</v>
       </c>
       <c r="G107">
-        <v>3.468</v>
+        <v>3.809</v>
       </c>
       <c r="H107">
-        <v>3.553</v>
+        <v>3.546</v>
       </c>
     </row>
     <row r="108" spans="1:8">

</xml_diff>

<commit_message>
Update ME1033 grades and correct formatting in CGPA results
</commit_message>
<xml_diff>
--- a/output/CGPA_Results.xlsx
+++ b/output/CGPA_Results.xlsx
@@ -310,6 +310,9 @@
     <t>PRABHARSHA H.W.D.</t>
   </si>
   <si>
+    <t>SANTHOSH S.</t>
+  </si>
+  <si>
     <t>MANATUNGA K.D.</t>
   </si>
   <si>
@@ -353,9 +356,6 @@
   </si>
   <si>
     <t>IMBULPITIYA B.N.</t>
-  </si>
-  <si>
-    <t>SANTHOSH S.</t>
   </si>
   <si>
     <t>AHAMED A.M.S.</t>
@@ -3088,25 +3088,25 @@
         <v>91</v>
       </c>
       <c r="B92">
-        <v>230395</v>
+        <v>230581</v>
       </c>
       <c r="C92" t="s">
         <v>98</v>
       </c>
       <c r="D92">
-        <v>3.85</v>
+        <v>3.835</v>
       </c>
       <c r="E92">
-        <v>3.656</v>
+        <v>3.629</v>
       </c>
       <c r="F92">
-        <v>3.334</v>
+        <v>3.509</v>
       </c>
       <c r="G92">
-        <v>3.945</v>
+        <v>3.809</v>
       </c>
       <c r="H92">
-        <v>3.676</v>
+        <v>3.683</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -3114,25 +3114,25 @@
         <v>92</v>
       </c>
       <c r="B93">
-        <v>230563</v>
+        <v>230395</v>
       </c>
       <c r="C93" t="s">
         <v>99</v>
       </c>
       <c r="D93">
-        <v>3.892</v>
+        <v>3.85</v>
       </c>
       <c r="E93">
-        <v>3.726</v>
+        <v>3.656</v>
       </c>
       <c r="F93">
-        <v>3.304</v>
+        <v>3.334</v>
       </c>
       <c r="G93">
-        <v>3.872</v>
+        <v>3.945</v>
       </c>
       <c r="H93">
-        <v>3.675</v>
+        <v>3.676</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -3140,25 +3140,25 @@
         <v>93</v>
       </c>
       <c r="B94">
-        <v>230650</v>
+        <v>230563</v>
       </c>
       <c r="C94" t="s">
         <v>100</v>
       </c>
       <c r="D94">
-        <v>4</v>
+        <v>3.892</v>
       </c>
       <c r="E94">
-        <v>3.708</v>
+        <v>3.726</v>
       </c>
       <c r="F94">
-        <v>3.373</v>
+        <v>3.304</v>
       </c>
       <c r="G94">
-        <v>3.722</v>
+        <v>3.872</v>
       </c>
       <c r="H94">
-        <v>3.668</v>
+        <v>3.675</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -3166,25 +3166,25 @@
         <v>94</v>
       </c>
       <c r="B95">
-        <v>230013</v>
+        <v>230650</v>
       </c>
       <c r="C95" t="s">
         <v>101</v>
       </c>
       <c r="D95">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E95">
-        <v>3.617</v>
+        <v>3.708</v>
       </c>
       <c r="F95">
-        <v>3.638</v>
+        <v>3.373</v>
       </c>
       <c r="G95">
-        <v>3.636</v>
+        <v>3.722</v>
       </c>
       <c r="H95">
-        <v>3.667</v>
+        <v>3.668</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -3192,7 +3192,7 @@
         <v>95</v>
       </c>
       <c r="B96">
-        <v>230229</v>
+        <v>230013</v>
       </c>
       <c r="C96" t="s">
         <v>102</v>
@@ -3201,16 +3201,16 @@
         <v>3.85</v>
       </c>
       <c r="E96">
-        <v>3.817</v>
+        <v>3.617</v>
       </c>
       <c r="F96">
-        <v>3.4</v>
+        <v>3.638</v>
       </c>
       <c r="G96">
-        <v>3.64</v>
+        <v>3.636</v>
       </c>
       <c r="H96">
-        <v>3.665</v>
+        <v>3.667</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -3218,25 +3218,25 @@
         <v>96</v>
       </c>
       <c r="B97">
-        <v>230458</v>
+        <v>230229</v>
       </c>
       <c r="C97" t="s">
         <v>103</v>
       </c>
       <c r="D97">
-        <v>3.957</v>
+        <v>3.85</v>
       </c>
       <c r="E97">
-        <v>3.713</v>
+        <v>3.817</v>
       </c>
       <c r="F97">
-        <v>3.465</v>
+        <v>3.4</v>
       </c>
       <c r="G97">
-        <v>3.627</v>
+        <v>3.64</v>
       </c>
       <c r="H97">
-        <v>3.662</v>
+        <v>3.665</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -3244,7 +3244,7 @@
         <v>97</v>
       </c>
       <c r="B98">
-        <v>230175</v>
+        <v>230458</v>
       </c>
       <c r="C98" t="s">
         <v>104</v>
@@ -3253,16 +3253,16 @@
         <v>3.957</v>
       </c>
       <c r="E98">
-        <v>3.695</v>
+        <v>3.713</v>
       </c>
       <c r="F98">
-        <v>3.404</v>
+        <v>3.465</v>
       </c>
       <c r="G98">
-        <v>3.629</v>
+        <v>3.627</v>
       </c>
       <c r="H98">
-        <v>3.64</v>
+        <v>3.662</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -3270,25 +3270,25 @@
         <v>98</v>
       </c>
       <c r="B99">
-        <v>230280</v>
+        <v>230175</v>
       </c>
       <c r="C99" t="s">
         <v>105</v>
       </c>
       <c r="D99">
-        <v>3.85</v>
+        <v>3.957</v>
       </c>
       <c r="E99">
-        <v>3.908</v>
+        <v>3.695</v>
       </c>
       <c r="F99">
-        <v>3.13</v>
+        <v>3.404</v>
       </c>
       <c r="G99">
-        <v>3.679</v>
+        <v>3.629</v>
       </c>
       <c r="H99">
-        <v>3.62</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="100" spans="1:8">
@@ -3296,25 +3296,25 @@
         <v>99</v>
       </c>
       <c r="B100">
-        <v>230208</v>
+        <v>230280</v>
       </c>
       <c r="C100" t="s">
         <v>106</v>
       </c>
       <c r="D100">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E100">
-        <v>3.617</v>
+        <v>3.908</v>
       </c>
       <c r="F100">
-        <v>3.46</v>
+        <v>3.13</v>
       </c>
       <c r="G100">
-        <v>3.513</v>
+        <v>3.679</v>
       </c>
       <c r="H100">
-        <v>3.61</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -3322,25 +3322,25 @@
         <v>100</v>
       </c>
       <c r="B101">
-        <v>230033</v>
+        <v>230208</v>
       </c>
       <c r="C101" t="s">
         <v>107</v>
       </c>
       <c r="D101">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E101">
-        <v>3.604</v>
+        <v>3.617</v>
       </c>
       <c r="F101">
-        <v>3.347</v>
+        <v>3.46</v>
       </c>
       <c r="G101">
-        <v>3.716</v>
+        <v>3.513</v>
       </c>
       <c r="H101">
-        <v>3.607</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="102" spans="1:8">
@@ -3348,25 +3348,25 @@
         <v>101</v>
       </c>
       <c r="B102">
-        <v>230636</v>
+        <v>230033</v>
       </c>
       <c r="C102" t="s">
         <v>108</v>
       </c>
       <c r="D102">
-        <v>3.892</v>
+        <v>3.85</v>
       </c>
       <c r="E102">
-        <v>3.578</v>
+        <v>3.604</v>
       </c>
       <c r="F102">
-        <v>3.278</v>
+        <v>3.347</v>
       </c>
       <c r="G102">
         <v>3.716</v>
       </c>
       <c r="H102">
-        <v>3.588</v>
+        <v>3.607</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -3374,25 +3374,25 @@
         <v>102</v>
       </c>
       <c r="B103">
-        <v>230520</v>
+        <v>230636</v>
       </c>
       <c r="C103" t="s">
         <v>109</v>
       </c>
       <c r="D103">
-        <v>3.85</v>
+        <v>3.892</v>
       </c>
       <c r="E103">
-        <v>3.726</v>
+        <v>3.578</v>
       </c>
       <c r="F103">
-        <v>3.43</v>
+        <v>3.278</v>
       </c>
       <c r="G103">
-        <v>3.452</v>
+        <v>3.716</v>
       </c>
       <c r="H103">
-        <v>3.585</v>
+        <v>3.588</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -3400,25 +3400,25 @@
         <v>103</v>
       </c>
       <c r="B104">
-        <v>230493</v>
+        <v>230520</v>
       </c>
       <c r="C104" t="s">
         <v>110</v>
       </c>
       <c r="D104">
-        <v>3.935</v>
+        <v>3.85</v>
       </c>
       <c r="E104">
-        <v>3.46</v>
+        <v>3.726</v>
       </c>
       <c r="F104">
-        <v>3.334</v>
+        <v>3.43</v>
       </c>
       <c r="G104">
-        <v>3.722</v>
+        <v>3.452</v>
       </c>
       <c r="H104">
-        <v>3.576</v>
+        <v>3.585</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -3426,25 +3426,25 @@
         <v>104</v>
       </c>
       <c r="B105">
-        <v>230564</v>
+        <v>230493</v>
       </c>
       <c r="C105" t="s">
         <v>111</v>
       </c>
       <c r="D105">
-        <v>3.871</v>
+        <v>3.935</v>
       </c>
       <c r="E105">
-        <v>3.421</v>
+        <v>3.46</v>
       </c>
       <c r="F105">
-        <v>3.221</v>
+        <v>3.334</v>
       </c>
       <c r="G105">
-        <v>3.837</v>
+        <v>3.722</v>
       </c>
       <c r="H105">
-        <v>3.56</v>
+        <v>3.576</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -3452,25 +3452,25 @@
         <v>105</v>
       </c>
       <c r="B106">
-        <v>230259</v>
+        <v>230564</v>
       </c>
       <c r="C106" t="s">
         <v>112</v>
       </c>
       <c r="D106">
-        <v>3.85</v>
+        <v>3.871</v>
       </c>
       <c r="E106">
-        <v>3.551</v>
+        <v>3.421</v>
       </c>
       <c r="F106">
-        <v>3.447</v>
+        <v>3.221</v>
       </c>
       <c r="G106">
-        <v>3.468</v>
+        <v>3.837</v>
       </c>
       <c r="H106">
-        <v>3.553</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -3478,25 +3478,25 @@
         <v>106</v>
       </c>
       <c r="B107">
-        <v>230581</v>
+        <v>230259</v>
       </c>
       <c r="C107" t="s">
         <v>113</v>
       </c>
       <c r="D107">
-        <v>3.735</v>
+        <v>3.85</v>
       </c>
       <c r="E107">
-        <v>3.629</v>
+        <v>3.551</v>
       </c>
       <c r="F107">
-        <v>3.014</v>
+        <v>3.447</v>
       </c>
       <c r="G107">
-        <v>3.809</v>
+        <v>3.468</v>
       </c>
       <c r="H107">
-        <v>3.546</v>
+        <v>3.553</v>
       </c>
     </row>
     <row r="108" spans="1:8">

</xml_diff>

<commit_message>
Update corrections and semester data; add new course EL2520 and adjust grades
</commit_message>
<xml_diff>
--- a/output/CGPA_Results.xlsx
+++ b/output/CGPA_Results.xlsx
@@ -238,15 +238,15 @@
     <t>WIJESINGHE U.G.S.K.D.</t>
   </si>
   <si>
+    <t>DISSANAYAKE R.K.T.</t>
+  </si>
+  <si>
     <t>RANATHUNGA R.J.K.O.H.</t>
   </si>
   <si>
     <t>WIJESINGHE W.A.P.W.</t>
   </si>
   <si>
-    <t>DISSANAYAKE R.K.T.</t>
-  </si>
-  <si>
     <t>ATHUKORALA U.R.</t>
   </si>
   <si>
@@ -346,10 +346,10 @@
     <t>THARUSHIKA G.K.E.</t>
   </si>
   <si>
+    <t>PIYUMAL N.P.P.</t>
+  </si>
+  <si>
     <t>RANASINGHE A.G.N.S.</t>
-  </si>
-  <si>
-    <t>PIYUMAL N.P.P.</t>
   </si>
   <si>
     <t>SAMARASEKARA S.M.R.P.</t>
@@ -2464,25 +2464,25 @@
         <v>67</v>
       </c>
       <c r="B68">
-        <v>230525</v>
+        <v>230164</v>
       </c>
       <c r="C68" t="s">
         <v>74</v>
       </c>
       <c r="D68">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E68">
-        <v>4</v>
+        <v>3.869</v>
       </c>
       <c r="F68">
-        <v>3.5</v>
+        <v>3.669</v>
       </c>
       <c r="G68">
-        <v>3.763</v>
+        <v>3.775</v>
       </c>
       <c r="H68">
-        <v>3.796</v>
+        <v>3.797</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -2490,25 +2490,25 @@
         <v>68</v>
       </c>
       <c r="B69">
-        <v>230727</v>
+        <v>230525</v>
       </c>
       <c r="C69" t="s">
         <v>75</v>
       </c>
       <c r="D69">
-        <v>3.785</v>
+        <v>4</v>
       </c>
       <c r="E69">
-        <v>3.888</v>
+        <v>4</v>
       </c>
       <c r="F69">
-        <v>3.54</v>
+        <v>3.5</v>
       </c>
       <c r="G69">
-        <v>3.918</v>
+        <v>3.763</v>
       </c>
       <c r="H69">
-        <v>3.795</v>
+        <v>3.796</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -2516,25 +2516,25 @@
         <v>69</v>
       </c>
       <c r="B70">
-        <v>230164</v>
+        <v>230727</v>
       </c>
       <c r="C70" t="s">
         <v>76</v>
       </c>
       <c r="D70">
-        <v>3.957</v>
+        <v>3.785</v>
       </c>
       <c r="E70">
-        <v>3.869</v>
+        <v>3.888</v>
       </c>
       <c r="F70">
-        <v>3.626</v>
+        <v>3.54</v>
       </c>
       <c r="G70">
-        <v>3.775</v>
+        <v>3.918</v>
       </c>
       <c r="H70">
-        <v>3.79</v>
+        <v>3.795</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -3400,25 +3400,25 @@
         <v>103</v>
       </c>
       <c r="B104">
-        <v>230520</v>
+        <v>230493</v>
       </c>
       <c r="C104" t="s">
         <v>110</v>
       </c>
       <c r="D104">
-        <v>3.85</v>
+        <v>3.935</v>
       </c>
       <c r="E104">
-        <v>3.726</v>
+        <v>3.46</v>
       </c>
       <c r="F104">
-        <v>3.43</v>
+        <v>3.373</v>
       </c>
       <c r="G104">
-        <v>3.452</v>
+        <v>3.722</v>
       </c>
       <c r="H104">
-        <v>3.585</v>
+        <v>3.587</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -3426,25 +3426,25 @@
         <v>104</v>
       </c>
       <c r="B105">
-        <v>230493</v>
+        <v>230520</v>
       </c>
       <c r="C105" t="s">
         <v>111</v>
       </c>
       <c r="D105">
-        <v>3.935</v>
+        <v>3.85</v>
       </c>
       <c r="E105">
-        <v>3.46</v>
+        <v>3.726</v>
       </c>
       <c r="F105">
-        <v>3.334</v>
+        <v>3.43</v>
       </c>
       <c r="G105">
-        <v>3.722</v>
+        <v>3.452</v>
       </c>
       <c r="H105">
-        <v>3.576</v>
+        <v>3.585</v>
       </c>
     </row>
     <row r="106" spans="1:8">

</xml_diff>

<commit_message>
Graph theory and corrections
</commit_message>
<xml_diff>
--- a/output/CGPA_Results.xlsx
+++ b/output/CGPA_Results.xlsx
@@ -79,12 +79,12 @@
     <t>WANIGASUNDARA W.M.H.</t>
   </si>
   <si>
+    <t>PERERA U.I.H.</t>
+  </si>
+  <si>
     <t>KUMARASINGHE M.N.</t>
   </si>
   <si>
-    <t>PERERA U.I.H.</t>
-  </si>
-  <si>
     <t>DE MEL D.J.</t>
   </si>
   <si>
@@ -115,12 +115,12 @@
     <t>DISSANAYAKA D.M.D.P.</t>
   </si>
   <si>
+    <t>BANDARA W.D.A.C.</t>
+  </si>
+  <si>
     <t>KEERAWELLA K.P.C.P.</t>
   </si>
   <si>
-    <t>BANDARA W.D.A.C.</t>
-  </si>
-  <si>
     <t>DISSANAYAKE G.R.G.K.</t>
   </si>
   <si>
@@ -154,78 +154,78 @@
     <t>AMARATHUNGE A.M.N.L.</t>
   </si>
   <si>
+    <t>WIJESEKARA W.A.G.S.</t>
+  </si>
+  <si>
+    <t>GUNATHUNGA U.A.</t>
+  </si>
+  <si>
+    <t>RATHEESHAN A.R.</t>
+  </si>
+  <si>
+    <t>JAYAWEERA N.S.</t>
+  </si>
+  <si>
+    <t>MUNASINGHE A.I.</t>
+  </si>
+  <si>
+    <t>UPEKSHANI T.S.</t>
+  </si>
+  <si>
+    <t>PEIRIS T.S.R.</t>
+  </si>
+  <si>
+    <t>WEERAKOON A.H.T.M.</t>
+  </si>
+  <si>
     <t>RASANJANA W.P.G.R.A.</t>
   </si>
   <si>
-    <t>WIJESEKARA W.A.G.S.</t>
-  </si>
-  <si>
-    <t>GUNATHUNGA U.A.</t>
-  </si>
-  <si>
-    <t>RATHEESHAN A.R.</t>
-  </si>
-  <si>
-    <t>JAYAWEERA N.S.</t>
-  </si>
-  <si>
-    <t>MUNASINGHE A.I.</t>
+    <t>PERERA H.A.J.I.</t>
   </si>
   <si>
     <t>DESHAN W.U.</t>
   </si>
   <si>
-    <t>UPEKSHANI T.S.</t>
-  </si>
-  <si>
-    <t>PEIRIS T.S.R.</t>
-  </si>
-  <si>
-    <t>WEERAKOON A.H.T.M.</t>
+    <t>PATHIRANA P.T.S.</t>
+  </si>
+  <si>
+    <t>PITIWADUGE D.N.</t>
   </si>
   <si>
     <t>KUMARA P.K.M.P.</t>
   </si>
   <si>
-    <t>PATHIRANA P.T.S.</t>
-  </si>
-  <si>
-    <t>PITIWADUGE D.N.</t>
+    <t>DILHAN W.A.</t>
+  </si>
+  <si>
+    <t>DHARMAKEERTHI P.K.G.C.L.</t>
+  </si>
+  <si>
+    <t>FERNANDO H.M.D.</t>
+  </si>
+  <si>
+    <t>KARUNANAYAKE A.H.D.</t>
+  </si>
+  <si>
+    <t>RAHMAN M.F.A.</t>
+  </si>
+  <si>
+    <t>TENNAKOON U.G.R.B.</t>
+  </si>
+  <si>
+    <t>AROSHANA H.A.P.</t>
   </si>
   <si>
     <t>PRIYADARSHANA S.A.D.</t>
   </si>
   <si>
-    <t>DILHAN W.A.</t>
-  </si>
-  <si>
-    <t>DHARMAKEERTHI P.K.G.C.L.</t>
-  </si>
-  <si>
-    <t>FERNANDO H.M.D.</t>
-  </si>
-  <si>
-    <t>KARUNANAYAKE A.H.D.</t>
-  </si>
-  <si>
-    <t>RAHMAN M.F.A.</t>
-  </si>
-  <si>
-    <t>TENNAKOON U.G.R.B.</t>
-  </si>
-  <si>
-    <t>AROSHANA H.A.P.</t>
-  </si>
-  <si>
     <t>GAMAGE SK</t>
   </si>
   <si>
     <t>PRISHMIKA H.W.N.</t>
   </si>
   <si>
-    <t>PERERA H.A.J.I.</t>
-  </si>
-  <si>
     <t>GUNASEKARA K.S.</t>
   </si>
   <si>
@@ -250,15 +250,15 @@
     <t>ATHUKORALA U.R.</t>
   </si>
   <si>
+    <t>UMAIR A.</t>
+  </si>
+  <si>
+    <t>MEEDENIYA M.M.H.</t>
+  </si>
+  <si>
     <t>DILHARA D.S.</t>
   </si>
   <si>
-    <t>UMAIR A.</t>
-  </si>
-  <si>
-    <t>MEEDENIYA M.M.H.</t>
-  </si>
-  <si>
     <t>ABISHEK L.</t>
   </si>
   <si>
@@ -268,60 +268,60 @@
     <t>SARUKA U.</t>
   </si>
   <si>
+    <t>INDUWARA M.L.A.S.</t>
+  </si>
+  <si>
+    <t>LENMINI B.L.W.</t>
+  </si>
+  <si>
+    <t>PERAMUNAGE D.S.</t>
+  </si>
+  <si>
+    <t>ARACHCHIGE M. A. D. T. S.</t>
+  </si>
+  <si>
+    <t>SHEHAN M.N.N.</t>
+  </si>
+  <si>
+    <t>ADHIKARI A.H.C.S.</t>
+  </si>
+  <si>
     <t>WITHANAGE G.D.N.</t>
   </si>
   <si>
-    <t>INDUWARA M.L.A.S.</t>
-  </si>
-  <si>
-    <t>LENMINI B.L.W.</t>
-  </si>
-  <si>
-    <t>PERAMUNAGE D.S.</t>
-  </si>
-  <si>
-    <t>ARACHCHIGE M. A. D. T. S.</t>
-  </si>
-  <si>
-    <t>SHEHAN M.N.N.</t>
-  </si>
-  <si>
-    <t>ADHIKARI A.H.C.S.</t>
-  </si>
-  <si>
     <t>KAUSHALYA R.G.S.P.</t>
   </si>
   <si>
     <t>ABEYWARDHANA T.C.W.</t>
   </si>
   <si>
+    <t>BANDARA K.M.N.D.</t>
+  </si>
+  <si>
+    <t>NIRMANI W.T.</t>
+  </si>
+  <si>
     <t>AYANAJA N.B.G.M.</t>
   </si>
   <si>
-    <t>BANDARA K.M.N.D.</t>
-  </si>
-  <si>
-    <t>NIRMANI W.T.</t>
+    <t>PRABHARSHA H.W.D.</t>
   </si>
   <si>
     <t>RANAWAKA R.A.G.K.</t>
   </si>
   <si>
-    <t>PRABHARSHA H.W.D.</t>
-  </si>
-  <si>
     <t>SANTHOSH S.</t>
   </si>
   <si>
+    <t>UBEYSEKARA V.T.T.</t>
+  </si>
+  <si>
     <t>MANATUNGA K.D.</t>
   </si>
   <si>
     <t>SAMARANAYAKA H.D.J.D.</t>
   </si>
   <si>
-    <t>UBEYSEKARA V.T.T.</t>
-  </si>
-  <si>
     <t>ABEYWARNA D.H.</t>
   </si>
   <si>
@@ -343,10 +343,10 @@
     <t>AMARASINGHE A.A.D.K.</t>
   </si>
   <si>
+    <t>PIYUMAL N.P.P.</t>
+  </si>
+  <si>
     <t>THARUSHIKA G.K.E.</t>
-  </si>
-  <si>
-    <t>PIYUMAL N.P.P.</t>
   </si>
   <si>
     <t>RANASINGHE A.G.N.S.</t>
@@ -1086,7 +1086,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>230355</v>
+        <v>230486</v>
       </c>
       <c r="C15" t="s">
         <v>21</v>
@@ -1098,13 +1098,13 @@
         <v>4</v>
       </c>
       <c r="F15">
-        <v>3.9</v>
+        <v>3.907</v>
       </c>
       <c r="G15">
         <v>4</v>
       </c>
       <c r="H15">
-        <v>3.971</v>
+        <v>3.972</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1112,7 +1112,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>230486</v>
+        <v>230355</v>
       </c>
       <c r="C16" t="s">
         <v>22</v>
@@ -1124,7 +1124,7 @@
         <v>4</v>
       </c>
       <c r="F16">
-        <v>3.907</v>
+        <v>3.9</v>
       </c>
       <c r="G16">
         <v>4</v>
@@ -1208,7 +1208,7 @@
         <v>4</v>
       </c>
       <c r="H19">
-        <v>3.966</v>
+        <v>3.967</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1312,7 +1312,7 @@
         <v>4</v>
       </c>
       <c r="H23">
-        <v>3.957</v>
+        <v>3.958</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1338,7 +1338,7 @@
         <v>4</v>
       </c>
       <c r="H24">
-        <v>3.954</v>
+        <v>3.955</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1364,7 +1364,7 @@
         <v>4</v>
       </c>
       <c r="H25">
-        <v>3.952</v>
+        <v>3.953</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1398,7 +1398,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>230332</v>
+        <v>230082</v>
       </c>
       <c r="C27" t="s">
         <v>33</v>
@@ -1410,10 +1410,10 @@
         <v>4</v>
       </c>
       <c r="F27">
-        <v>3.79</v>
+        <v>3.96</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>3.873</v>
       </c>
       <c r="H27">
         <v>3.951</v>
@@ -1424,7 +1424,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>230082</v>
+        <v>230332</v>
       </c>
       <c r="C28" t="s">
         <v>34</v>
@@ -1436,13 +1436,13 @@
         <v>4</v>
       </c>
       <c r="F28">
-        <v>3.96</v>
+        <v>3.79</v>
       </c>
       <c r="G28">
-        <v>3.862</v>
+        <v>4</v>
       </c>
       <c r="H28">
-        <v>3.95</v>
+        <v>3.951</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1673,10 +1673,10 @@
         <v>3.704</v>
       </c>
       <c r="G37">
-        <v>3.945</v>
+        <v>3.925</v>
       </c>
       <c r="H37">
-        <v>3.902</v>
+        <v>3.897</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1736,25 +1736,25 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>230536</v>
+        <v>230724</v>
       </c>
       <c r="C40" t="s">
         <v>46</v>
       </c>
       <c r="D40">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E40">
-        <v>3.96</v>
+        <v>3.869</v>
       </c>
       <c r="F40">
         <v>3.847</v>
       </c>
       <c r="G40">
-        <v>3.833</v>
+        <v>3.89</v>
       </c>
       <c r="H40">
-        <v>3.892</v>
+        <v>3.891</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -1762,25 +1762,25 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>230724</v>
+        <v>230218</v>
       </c>
       <c r="C41" t="s">
         <v>47</v>
       </c>
       <c r="D41">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E41">
-        <v>3.869</v>
+        <v>3.811</v>
       </c>
       <c r="F41">
-        <v>3.847</v>
+        <v>3.825</v>
       </c>
       <c r="G41">
-        <v>3.89</v>
+        <v>4</v>
       </c>
       <c r="H41">
-        <v>3.891</v>
+        <v>3.885</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -1788,7 +1788,7 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>230218</v>
+        <v>230539</v>
       </c>
       <c r="C42" t="s">
         <v>48</v>
@@ -1797,16 +1797,16 @@
         <v>3.935</v>
       </c>
       <c r="E42">
-        <v>3.811</v>
+        <v>4</v>
       </c>
       <c r="F42">
-        <v>3.825</v>
+        <v>3.652</v>
       </c>
       <c r="G42">
-        <v>4</v>
+        <v>3.964</v>
       </c>
       <c r="H42">
-        <v>3.885</v>
+        <v>3.884</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -1814,7 +1814,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>230539</v>
+        <v>230300</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
@@ -1826,13 +1826,13 @@
         <v>4</v>
       </c>
       <c r="F43">
-        <v>3.652</v>
+        <v>3.713</v>
       </c>
       <c r="G43">
-        <v>3.964</v>
+        <v>3.89</v>
       </c>
       <c r="H43">
-        <v>3.884</v>
+        <v>3.879</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -1840,22 +1840,22 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>230300</v>
+        <v>230417</v>
       </c>
       <c r="C44" t="s">
         <v>50</v>
       </c>
       <c r="D44">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E44">
-        <v>4</v>
+        <v>3.939</v>
       </c>
       <c r="F44">
-        <v>3.713</v>
+        <v>3.804</v>
       </c>
       <c r="G44">
-        <v>3.89</v>
+        <v>3.818</v>
       </c>
       <c r="H44">
         <v>3.879</v>
@@ -1866,25 +1866,25 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>230417</v>
+        <v>230659</v>
       </c>
       <c r="C45" t="s">
         <v>51</v>
       </c>
       <c r="D45">
-        <v>4</v>
+        <v>3.857</v>
       </c>
       <c r="E45">
-        <v>3.939</v>
+        <v>3.869</v>
       </c>
       <c r="F45">
         <v>3.804</v>
       </c>
       <c r="G45">
-        <v>3.818</v>
+        <v>3.945</v>
       </c>
       <c r="H45">
-        <v>3.879</v>
+        <v>3.869</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -1892,7 +1892,7 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>230130</v>
+        <v>230470</v>
       </c>
       <c r="C46" t="s">
         <v>52</v>
@@ -1901,16 +1901,16 @@
         <v>4</v>
       </c>
       <c r="E46">
-        <v>3.96</v>
+        <v>4</v>
       </c>
       <c r="F46">
-        <v>3.714</v>
+        <v>3.526</v>
       </c>
       <c r="G46">
-        <v>3.863</v>
+        <v>4</v>
       </c>
       <c r="H46">
-        <v>3.876</v>
+        <v>3.867</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -1918,25 +1918,25 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>230659</v>
+        <v>230689</v>
       </c>
       <c r="C47" t="s">
         <v>53</v>
       </c>
       <c r="D47">
-        <v>3.857</v>
+        <v>4</v>
       </c>
       <c r="E47">
-        <v>3.869</v>
+        <v>4</v>
       </c>
       <c r="F47">
-        <v>3.804</v>
+        <v>3.771</v>
       </c>
       <c r="G47">
-        <v>3.945</v>
+        <v>3.745</v>
       </c>
       <c r="H47">
-        <v>3.869</v>
+        <v>3.867</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -1944,25 +1944,25 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>230470</v>
+        <v>230536</v>
       </c>
       <c r="C48" t="s">
         <v>54</v>
       </c>
       <c r="D48">
-        <v>4</v>
+        <v>3.957</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>3.96</v>
       </c>
       <c r="F48">
-        <v>3.526</v>
+        <v>3.847</v>
       </c>
       <c r="G48">
-        <v>4</v>
+        <v>3.746</v>
       </c>
       <c r="H48">
-        <v>3.867</v>
+        <v>3.865</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -1970,25 +1970,25 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>230689</v>
+        <v>230477</v>
       </c>
       <c r="C49" t="s">
         <v>55</v>
       </c>
       <c r="D49">
-        <v>4</v>
+        <v>3.935</v>
       </c>
       <c r="E49">
-        <v>4</v>
+        <v>3.908</v>
       </c>
       <c r="F49">
-        <v>3.771</v>
+        <v>3.873</v>
       </c>
       <c r="G49">
-        <v>3.745</v>
+        <v>3.77</v>
       </c>
       <c r="H49">
-        <v>3.867</v>
+        <v>3.864</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -1996,25 +1996,25 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>230353</v>
+        <v>230130</v>
       </c>
       <c r="C50" t="s">
         <v>56</v>
       </c>
       <c r="D50">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="E50">
         <v>3.96</v>
       </c>
       <c r="F50">
-        <v>3.613</v>
+        <v>3.714</v>
       </c>
       <c r="G50">
-        <v>4</v>
+        <v>3.816</v>
       </c>
       <c r="H50">
-        <v>3.863</v>
+        <v>3.862</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2074,25 +2074,25 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>230502</v>
+        <v>230353</v>
       </c>
       <c r="C53" t="s">
         <v>59</v>
       </c>
       <c r="D53">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="E53">
-        <v>3.947</v>
+        <v>3.96</v>
       </c>
       <c r="F53">
-        <v>3.586</v>
+        <v>3.613</v>
       </c>
       <c r="G53">
-        <v>3.945</v>
+        <v>3.975</v>
       </c>
       <c r="H53">
-        <v>3.854</v>
+        <v>3.859</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2282,25 +2282,25 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>230195</v>
+        <v>230502</v>
       </c>
       <c r="C61" t="s">
         <v>67</v>
       </c>
       <c r="D61">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="E61">
-        <v>3.791</v>
+        <v>3.947</v>
       </c>
       <c r="F61">
-        <v>3.678</v>
+        <v>3.586</v>
       </c>
       <c r="G61">
-        <v>3.925</v>
+        <v>3.841</v>
       </c>
       <c r="H61">
-        <v>3.826</v>
+        <v>3.827</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2308,7 +2308,7 @@
         <v>61</v>
       </c>
       <c r="B62">
-        <v>230500</v>
+        <v>230195</v>
       </c>
       <c r="C62" t="s">
         <v>68</v>
@@ -2317,16 +2317,16 @@
         <v>3.957</v>
       </c>
       <c r="E62">
-        <v>3.908</v>
+        <v>3.791</v>
       </c>
       <c r="F62">
         <v>3.678</v>
       </c>
       <c r="G62">
-        <v>3.809</v>
+        <v>3.925</v>
       </c>
       <c r="H62">
-        <v>3.825</v>
+        <v>3.826</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2334,25 +2334,25 @@
         <v>62</v>
       </c>
       <c r="B63">
-        <v>230477</v>
+        <v>230500</v>
       </c>
       <c r="C63" t="s">
         <v>69</v>
       </c>
       <c r="D63">
-        <v>3.935</v>
+        <v>3.957</v>
       </c>
       <c r="E63">
-        <v>3.817</v>
+        <v>3.908</v>
       </c>
       <c r="F63">
-        <v>3.873</v>
+        <v>3.678</v>
       </c>
       <c r="G63">
-        <v>3.704</v>
+        <v>3.809</v>
       </c>
       <c r="H63">
-        <v>3.82</v>
+        <v>3.825</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2568,25 +2568,25 @@
         <v>71</v>
       </c>
       <c r="B72">
-        <v>230147</v>
+        <v>230654</v>
       </c>
       <c r="C72" t="s">
         <v>78</v>
       </c>
       <c r="D72">
-        <v>3.892</v>
+        <v>3.935</v>
       </c>
       <c r="E72">
-        <v>3.817</v>
+        <v>3.839</v>
       </c>
       <c r="F72">
-        <v>3.508</v>
+        <v>3.591</v>
       </c>
       <c r="G72">
-        <v>3.945</v>
+        <v>3.799</v>
       </c>
       <c r="H72">
-        <v>3.778</v>
+        <v>3.776</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -2594,25 +2594,25 @@
         <v>72</v>
       </c>
       <c r="B73">
-        <v>230654</v>
+        <v>230407</v>
       </c>
       <c r="C73" t="s">
         <v>79</v>
       </c>
       <c r="D73">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E73">
-        <v>3.839</v>
+        <v>3.756</v>
       </c>
       <c r="F73">
-        <v>3.591</v>
+        <v>3.508</v>
       </c>
       <c r="G73">
-        <v>3.799</v>
+        <v>3.904</v>
       </c>
       <c r="H73">
-        <v>3.776</v>
+        <v>3.768</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -2620,25 +2620,25 @@
         <v>73</v>
       </c>
       <c r="B74">
-        <v>230407</v>
+        <v>230147</v>
       </c>
       <c r="C74" t="s">
         <v>80</v>
       </c>
       <c r="D74">
-        <v>4</v>
+        <v>3.892</v>
       </c>
       <c r="E74">
-        <v>3.756</v>
+        <v>3.817</v>
       </c>
       <c r="F74">
         <v>3.508</v>
       </c>
       <c r="G74">
-        <v>3.904</v>
+        <v>3.891</v>
       </c>
       <c r="H74">
-        <v>3.768</v>
+        <v>3.766</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -2713,10 +2713,10 @@
         <v>3.543</v>
       </c>
       <c r="G77">
-        <v>3.679</v>
+        <v>3.68</v>
       </c>
       <c r="H77">
-        <v>3.761</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -2724,25 +2724,25 @@
         <v>77</v>
       </c>
       <c r="B78">
-        <v>230735</v>
+        <v>230261</v>
       </c>
       <c r="C78" t="s">
         <v>84</v>
       </c>
       <c r="D78">
-        <v>3.935</v>
+        <v>4</v>
       </c>
       <c r="E78">
-        <v>3.786</v>
+        <v>3.747</v>
       </c>
       <c r="F78">
-        <v>3.399</v>
+        <v>3.458</v>
       </c>
       <c r="G78">
-        <v>4</v>
+        <v>3.945</v>
       </c>
       <c r="H78">
-        <v>3.76</v>
+        <v>3.759</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -2750,19 +2750,19 @@
         <v>78</v>
       </c>
       <c r="B79">
-        <v>230261</v>
+        <v>230375</v>
       </c>
       <c r="C79" t="s">
         <v>85</v>
       </c>
       <c r="D79">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E79">
-        <v>3.747</v>
+        <v>3.686</v>
       </c>
       <c r="F79">
-        <v>3.458</v>
+        <v>3.599</v>
       </c>
       <c r="G79">
         <v>3.945</v>
@@ -2776,22 +2776,22 @@
         <v>79</v>
       </c>
       <c r="B80">
-        <v>230375</v>
+        <v>230473</v>
       </c>
       <c r="C80" t="s">
         <v>86</v>
       </c>
       <c r="D80">
-        <v>3.85</v>
+        <v>3.892</v>
       </c>
       <c r="E80">
-        <v>3.686</v>
+        <v>3.908</v>
       </c>
       <c r="F80">
-        <v>3.599</v>
+        <v>3.443</v>
       </c>
       <c r="G80">
-        <v>3.945</v>
+        <v>3.849</v>
       </c>
       <c r="H80">
         <v>3.759</v>
@@ -2802,25 +2802,25 @@
         <v>80</v>
       </c>
       <c r="B81">
-        <v>230473</v>
+        <v>230052</v>
       </c>
       <c r="C81" t="s">
         <v>87</v>
       </c>
       <c r="D81">
-        <v>3.892</v>
+        <v>3.75</v>
       </c>
       <c r="E81">
-        <v>3.908</v>
+        <v>3.844</v>
       </c>
       <c r="F81">
-        <v>3.443</v>
+        <v>3.63</v>
       </c>
       <c r="G81">
-        <v>3.849</v>
+        <v>3.768</v>
       </c>
       <c r="H81">
-        <v>3.759</v>
+        <v>3.756</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -2828,25 +2828,25 @@
         <v>81</v>
       </c>
       <c r="B82">
-        <v>230052</v>
+        <v>230613</v>
       </c>
       <c r="C82" t="s">
         <v>88</v>
       </c>
       <c r="D82">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="E82">
-        <v>3.844</v>
+        <v>3.947</v>
       </c>
       <c r="F82">
-        <v>3.63</v>
+        <v>3.699</v>
       </c>
       <c r="G82">
-        <v>3.768</v>
+        <v>3.445</v>
       </c>
       <c r="H82">
-        <v>3.756</v>
+        <v>3.752</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -2854,25 +2854,25 @@
         <v>82</v>
       </c>
       <c r="B83">
-        <v>230613</v>
+        <v>230017</v>
       </c>
       <c r="C83" t="s">
         <v>89</v>
       </c>
       <c r="D83">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="E83">
         <v>3.947</v>
       </c>
       <c r="F83">
-        <v>3.699</v>
+        <v>3.441</v>
       </c>
       <c r="G83">
-        <v>3.445</v>
+        <v>3.79</v>
       </c>
       <c r="H83">
-        <v>3.752</v>
+        <v>3.751</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -2880,25 +2880,25 @@
         <v>83</v>
       </c>
       <c r="B84">
-        <v>230017</v>
+        <v>230735</v>
       </c>
       <c r="C84" t="s">
         <v>90</v>
       </c>
       <c r="D84">
-        <v>3.9</v>
+        <v>3.935</v>
       </c>
       <c r="E84">
-        <v>3.947</v>
+        <v>3.786</v>
       </c>
       <c r="F84">
-        <v>3.441</v>
+        <v>3.399</v>
       </c>
       <c r="G84">
-        <v>3.79</v>
+        <v>3.941</v>
       </c>
       <c r="H84">
-        <v>3.751</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -2921,10 +2921,10 @@
         <v>3.765</v>
       </c>
       <c r="G85">
-        <v>3.681</v>
+        <v>3.708</v>
       </c>
       <c r="H85">
-        <v>3.741</v>
+        <v>3.747</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -2958,22 +2958,22 @@
         <v>86</v>
       </c>
       <c r="B87">
-        <v>230065</v>
+        <v>230077</v>
       </c>
       <c r="C87" t="s">
         <v>93</v>
       </c>
       <c r="D87">
-        <v>3.892</v>
+        <v>3.785</v>
       </c>
       <c r="E87">
-        <v>3.83</v>
+        <v>3.733</v>
       </c>
       <c r="F87">
-        <v>3.347</v>
+        <v>3.619</v>
       </c>
       <c r="G87">
-        <v>3.945</v>
+        <v>3.822</v>
       </c>
       <c r="H87">
         <v>3.736</v>
@@ -2984,7 +2984,7 @@
         <v>87</v>
       </c>
       <c r="B88">
-        <v>230077</v>
+        <v>230444</v>
       </c>
       <c r="C88" t="s">
         <v>94</v>
@@ -2993,16 +2993,16 @@
         <v>3.785</v>
       </c>
       <c r="E88">
-        <v>3.733</v>
+        <v>3.596</v>
       </c>
       <c r="F88">
-        <v>3.619</v>
+        <v>3.757</v>
       </c>
       <c r="G88">
         <v>3.822</v>
       </c>
       <c r="H88">
-        <v>3.736</v>
+        <v>3.727</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -3010,25 +3010,25 @@
         <v>88</v>
       </c>
       <c r="B89">
-        <v>230444</v>
+        <v>230065</v>
       </c>
       <c r="C89" t="s">
         <v>95</v>
       </c>
       <c r="D89">
-        <v>3.785</v>
+        <v>3.892</v>
       </c>
       <c r="E89">
-        <v>3.596</v>
+        <v>3.83</v>
       </c>
       <c r="F89">
-        <v>3.757</v>
+        <v>3.347</v>
       </c>
       <c r="G89">
-        <v>3.822</v>
+        <v>3.866</v>
       </c>
       <c r="H89">
-        <v>3.727</v>
+        <v>3.719</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -3036,25 +3036,25 @@
         <v>89</v>
       </c>
       <c r="B90">
-        <v>230527</v>
+        <v>230495</v>
       </c>
       <c r="C90" t="s">
         <v>96</v>
       </c>
       <c r="D90">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="E90">
-        <v>3.83</v>
+        <v>3.869</v>
       </c>
       <c r="F90">
-        <v>3.339</v>
+        <v>3.443</v>
       </c>
       <c r="G90">
-        <v>3.849</v>
+        <v>3.758</v>
       </c>
       <c r="H90">
-        <v>3.726</v>
+        <v>3.717</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -3062,25 +3062,25 @@
         <v>90</v>
       </c>
       <c r="B91">
-        <v>230495</v>
+        <v>230527</v>
       </c>
       <c r="C91" t="s">
         <v>97</v>
       </c>
       <c r="D91">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E91">
-        <v>3.869</v>
+        <v>3.83</v>
       </c>
       <c r="F91">
-        <v>3.443</v>
+        <v>3.339</v>
       </c>
       <c r="G91">
-        <v>3.758</v>
+        <v>3.779</v>
       </c>
       <c r="H91">
-        <v>3.717</v>
+        <v>3.709</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -3114,25 +3114,25 @@
         <v>92</v>
       </c>
       <c r="B93">
-        <v>230395</v>
+        <v>230650</v>
       </c>
       <c r="C93" t="s">
         <v>99</v>
       </c>
       <c r="D93">
-        <v>3.85</v>
+        <v>4</v>
       </c>
       <c r="E93">
-        <v>3.656</v>
+        <v>3.747</v>
       </c>
       <c r="F93">
-        <v>3.334</v>
+        <v>3.373</v>
       </c>
       <c r="G93">
-        <v>3.945</v>
+        <v>3.722</v>
       </c>
       <c r="H93">
-        <v>3.676</v>
+        <v>3.679</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -3140,25 +3140,25 @@
         <v>93</v>
       </c>
       <c r="B94">
-        <v>230563</v>
+        <v>230395</v>
       </c>
       <c r="C94" t="s">
         <v>100</v>
       </c>
       <c r="D94">
-        <v>3.892</v>
+        <v>3.85</v>
       </c>
       <c r="E94">
-        <v>3.726</v>
+        <v>3.656</v>
       </c>
       <c r="F94">
-        <v>3.304</v>
+        <v>3.334</v>
       </c>
       <c r="G94">
-        <v>3.872</v>
+        <v>3.945</v>
       </c>
       <c r="H94">
-        <v>3.675</v>
+        <v>3.676</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -3166,25 +3166,25 @@
         <v>94</v>
       </c>
       <c r="B95">
-        <v>230650</v>
+        <v>230563</v>
       </c>
       <c r="C95" t="s">
         <v>101</v>
       </c>
       <c r="D95">
-        <v>4</v>
+        <v>3.892</v>
       </c>
       <c r="E95">
-        <v>3.708</v>
+        <v>3.726</v>
       </c>
       <c r="F95">
-        <v>3.373</v>
+        <v>3.304</v>
       </c>
       <c r="G95">
-        <v>3.722</v>
+        <v>3.872</v>
       </c>
       <c r="H95">
-        <v>3.668</v>
+        <v>3.675</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -3207,7 +3207,7 @@
         <v>3.638</v>
       </c>
       <c r="G96">
-        <v>3.636</v>
+        <v>3.641</v>
       </c>
       <c r="H96">
         <v>3.667</v>
@@ -3233,7 +3233,7 @@
         <v>3.4</v>
       </c>
       <c r="G97">
-        <v>3.64</v>
+        <v>3.645</v>
       </c>
       <c r="H97">
         <v>3.665</v>
@@ -3259,10 +3259,10 @@
         <v>3.465</v>
       </c>
       <c r="G98">
-        <v>3.627</v>
+        <v>3.6</v>
       </c>
       <c r="H98">
-        <v>3.662</v>
+        <v>3.653</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -3374,25 +3374,25 @@
         <v>102</v>
       </c>
       <c r="B103">
-        <v>230636</v>
+        <v>230493</v>
       </c>
       <c r="C103" t="s">
         <v>109</v>
       </c>
       <c r="D103">
-        <v>3.892</v>
+        <v>3.935</v>
       </c>
       <c r="E103">
-        <v>3.578</v>
+        <v>3.46</v>
       </c>
       <c r="F103">
-        <v>3.278</v>
+        <v>3.373</v>
       </c>
       <c r="G103">
-        <v>3.716</v>
+        <v>3.777</v>
       </c>
       <c r="H103">
-        <v>3.588</v>
+        <v>3.602</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -3400,25 +3400,25 @@
         <v>103</v>
       </c>
       <c r="B104">
-        <v>230493</v>
+        <v>230636</v>
       </c>
       <c r="C104" t="s">
         <v>110</v>
       </c>
       <c r="D104">
-        <v>3.935</v>
+        <v>3.892</v>
       </c>
       <c r="E104">
-        <v>3.46</v>
+        <v>3.578</v>
       </c>
       <c r="F104">
-        <v>3.373</v>
+        <v>3.278</v>
       </c>
       <c r="G104">
-        <v>3.722</v>
+        <v>3.716</v>
       </c>
       <c r="H104">
-        <v>3.587</v>
+        <v>3.588</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -3519,10 +3519,10 @@
         <v>3.004</v>
       </c>
       <c r="G108">
-        <v>3.427</v>
+        <v>3.333</v>
       </c>
       <c r="H108">
-        <v>3.526</v>
+        <v>3.497</v>
       </c>
     </row>
     <row r="109" spans="1:8">

</xml_diff>